<commit_message>
Update dashboard and reports with 9-14-BKG+PD booking data
Regenerated from "9-14-BKG+PD.xls": 1041 BK No outstanding (2658
containers) — a much larger dataset than prior runs, including
2 rows flagged for missing Pickup Name and two new depots
(UNITHAI CONTAINER TERMINAL, ICD LKT - Esco Ladkrabang GATE 2).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AI$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AI$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI6"/>
+  <dimension ref="A1:AI17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -826,7 +826,7 @@
         <v>0</v>
       </c>
       <c r="Y3" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z3" s="4">
         <f>SUM(O3:W3)-X3</f>
@@ -872,7 +872,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802484</t>
+          <t>HASLS22260701913</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -898,364 +898,1924 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx2 </t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>20260918</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>YUSEN LOGISTICS (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>MAKITA MANUFACTURING (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELECTRIC POWER TOOLS </t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>good, clean, dry, no leak, no hole, no smell, no oil container</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pickup : 2026-09-18, Return : 2026-09-20 (1ST RTN 20/09 W/O  RENT) 
+ ** PLEASE CHECK OPEN GATE BEFORE RETURN CNTR **
+</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="4">
+        <f>SUM(O4:W4)-X4</f>
+        <v/>
+      </c>
+      <c r="AA4" s="4">
+        <f>MAX(0,O4-MAX(0,X4))</f>
+        <v/>
+      </c>
+      <c r="AB4" s="4">
+        <f>MAX(0,P4-MAX(0,X4-SUM(O4:O4)))</f>
+        <v/>
+      </c>
+      <c r="AC4" s="4">
+        <f>MAX(0,Q4-MAX(0,X4-SUM(O4:P4)))</f>
+        <v/>
+      </c>
+      <c r="AD4" s="4">
+        <f>MAX(0,R4-MAX(0,X4-SUM(O4:Q4)))</f>
+        <v/>
+      </c>
+      <c r="AE4" s="4">
+        <f>MAX(0,S4-MAX(0,X4-SUM(O4:R4)))</f>
+        <v/>
+      </c>
+      <c r="AF4" s="4">
+        <f>MAX(0,T4-MAX(0,X4-SUM(O4:S4)))</f>
+        <v/>
+      </c>
+      <c r="AG4" s="4">
+        <f>MAX(0,U4-MAX(0,X4-SUM(O4:T4)))</f>
+        <v/>
+      </c>
+      <c r="AH4" s="4">
+        <f>MAX(0,V4-MAX(0,X4-SUM(O4:U4)))</f>
+        <v/>
+      </c>
+      <c r="AI4" s="4">
+        <f>MAX(0,W4-MAX(0,X4-SUM(O4:V4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260801508</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>SWSP</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>202610020330</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>KRPTK</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx40 </t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>20260921</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>SAMSUNG SDS GLOBAL SCL (THAILAND) CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>REFRIGERATOR</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>*No containers with cut and patch marks inside*
+GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Pickup : 2026-09-21, Return : 2026-09-22</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="4">
+        <f>SUM(O5:W5)-X5</f>
+        <v/>
+      </c>
+      <c r="AA5" s="4">
+        <f>MAX(0,O5-MAX(0,X5))</f>
+        <v/>
+      </c>
+      <c r="AB5" s="4">
+        <f>MAX(0,P5-MAX(0,X5-SUM(O5:O5)))</f>
+        <v/>
+      </c>
+      <c r="AC5" s="4">
+        <f>MAX(0,Q5-MAX(0,X5-SUM(O5:P5)))</f>
+        <v/>
+      </c>
+      <c r="AD5" s="4">
+        <f>MAX(0,R5-MAX(0,X5-SUM(O5:Q5)))</f>
+        <v/>
+      </c>
+      <c r="AE5" s="4">
+        <f>MAX(0,S5-MAX(0,X5-SUM(O5:R5)))</f>
+        <v/>
+      </c>
+      <c r="AF5" s="4">
+        <f>MAX(0,T5-MAX(0,X5-SUM(O5:S5)))</f>
+        <v/>
+      </c>
+      <c r="AG5" s="4">
+        <f>MAX(0,U5-MAX(0,X5-SUM(O5:T5)))</f>
+        <v/>
+      </c>
+      <c r="AH5" s="4">
+        <f>MAX(0,V5-MAX(0,X5-SUM(O5:U5)))</f>
+        <v/>
+      </c>
+      <c r="AI5" s="4">
+        <f>MAX(0,W5-MAX(0,X5-SUM(O5:V5)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260801889</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>ICVY</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>2607S</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>202609210300</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>IDJKT</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>ILOGS GLOBAL CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>MAJESTY HOLDINGS (ASIA) CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>Pickup : 2026-09-14, Return : 2026-09-14</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="4">
+        <f>SUM(O6:W6)-X6</f>
+        <v/>
+      </c>
+      <c r="AA6" s="4">
+        <f>MAX(0,O6-MAX(0,X6))</f>
+        <v/>
+      </c>
+      <c r="AB6" s="4">
+        <f>MAX(0,P6-MAX(0,X6-SUM(O6:O6)))</f>
+        <v/>
+      </c>
+      <c r="AC6" s="4">
+        <f>MAX(0,Q6-MAX(0,X6-SUM(O6:P6)))</f>
+        <v/>
+      </c>
+      <c r="AD6" s="4">
+        <f>MAX(0,R6-MAX(0,X6-SUM(O6:Q6)))</f>
+        <v/>
+      </c>
+      <c r="AE6" s="4">
+        <f>MAX(0,S6-MAX(0,X6-SUM(O6:R6)))</f>
+        <v/>
+      </c>
+      <c r="AF6" s="4">
+        <f>MAX(0,T6-MAX(0,X6-SUM(O6:S6)))</f>
+        <v/>
+      </c>
+      <c r="AG6" s="4">
+        <f>MAX(0,U6-MAX(0,X6-SUM(O6:T6)))</f>
+        <v/>
+      </c>
+      <c r="AH6" s="4">
+        <f>MAX(0,V6-MAX(0,X6-SUM(O6:U6)))</f>
+        <v/>
+      </c>
+      <c r="AI6" s="4">
+        <f>MAX(0,W6-MAX(0,X6-SUM(O6:V6)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802124</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>DJCF</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>0152N</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>202610110100</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>KRPTK</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx16 </t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>20261002</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>SAMSUNG SDS GLOBAL SCL (THAILAND) CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>REFRIGERATOR</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>*No containers with cut and patch marks inside*
+GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Pickup : 2026-10-02, Return : 2026-10-04</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="4">
+        <f>SUM(O7:W7)-X7</f>
+        <v/>
+      </c>
+      <c r="AA7" s="4">
+        <f>MAX(0,O7-MAX(0,X7))</f>
+        <v/>
+      </c>
+      <c r="AB7" s="4">
+        <f>MAX(0,P7-MAX(0,X7-SUM(O7:O7)))</f>
+        <v/>
+      </c>
+      <c r="AC7" s="4">
+        <f>MAX(0,Q7-MAX(0,X7-SUM(O7:P7)))</f>
+        <v/>
+      </c>
+      <c r="AD7" s="4">
+        <f>MAX(0,R7-MAX(0,X7-SUM(O7:Q7)))</f>
+        <v/>
+      </c>
+      <c r="AE7" s="4">
+        <f>MAX(0,S7-MAX(0,X7-SUM(O7:R7)))</f>
+        <v/>
+      </c>
+      <c r="AF7" s="4">
+        <f>MAX(0,T7-MAX(0,X7-SUM(O7:S7)))</f>
+        <v/>
+      </c>
+      <c r="AG7" s="4">
+        <f>MAX(0,U7-MAX(0,X7-SUM(O7:T7)))</f>
+        <v/>
+      </c>
+      <c r="AH7" s="4">
+        <f>MAX(0,V7-MAX(0,X7-SUM(O7:U7)))</f>
+        <v/>
+      </c>
+      <c r="AI7" s="4">
+        <f>MAX(0,W7-MAX(0,X7-SUM(O7:V7)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802276</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>202610011100</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>TWKEL</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>20260924</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>COSMO LOGISTICS CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>L. LIGHTING GLASS CO., LTD.</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>GLASS TUBES FOR ELECTRIC LIGHTING</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Pickup : 2026-09-24, Return : 2026-09-25 // CLS TIME 27/09 @23.59 
+ ** PLEASE CHECK OPEN GATE BEFORE RETURN CNTR **</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="4">
+        <f>SUM(O8:W8)-X8</f>
+        <v/>
+      </c>
+      <c r="AA8" s="4">
+        <f>MAX(0,O8-MAX(0,X8))</f>
+        <v/>
+      </c>
+      <c r="AB8" s="4">
+        <f>MAX(0,P8-MAX(0,X8-SUM(O8:O8)))</f>
+        <v/>
+      </c>
+      <c r="AC8" s="4">
+        <f>MAX(0,Q8-MAX(0,X8-SUM(O8:P8)))</f>
+        <v/>
+      </c>
+      <c r="AD8" s="4">
+        <f>MAX(0,R8-MAX(0,X8-SUM(O8:Q8)))</f>
+        <v/>
+      </c>
+      <c r="AE8" s="4">
+        <f>MAX(0,S8-MAX(0,X8-SUM(O8:R8)))</f>
+        <v/>
+      </c>
+      <c r="AF8" s="4">
+        <f>MAX(0,T8-MAX(0,X8-SUM(O8:S8)))</f>
+        <v/>
+      </c>
+      <c r="AG8" s="4">
+        <f>MAX(0,U8-MAX(0,X8-SUM(O8:T8)))</f>
+        <v/>
+      </c>
+      <c r="AH8" s="4">
+        <f>MAX(0,V8-MAX(0,X8-SUM(O8:U8)))</f>
+        <v/>
+      </c>
+      <c r="AI8" s="4">
+        <f>MAX(0,W8-MAX(0,X8-SUM(O8:V8)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802290</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>SWIC</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>202609220500</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>KRPUS</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>ALUCON PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>ALUCON PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>EMPTY ALUMINIUM TUBES</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Pickup : 2026-09-17, Return : 2026-09-19</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="4">
+        <f>SUM(O9:W9)-X9</f>
+        <v/>
+      </c>
+      <c r="AA9" s="4">
+        <f>MAX(0,O9-MAX(0,X9))</f>
+        <v/>
+      </c>
+      <c r="AB9" s="4">
+        <f>MAX(0,P9-MAX(0,X9-SUM(O9:O9)))</f>
+        <v/>
+      </c>
+      <c r="AC9" s="4">
+        <f>MAX(0,Q9-MAX(0,X9-SUM(O9:P9)))</f>
+        <v/>
+      </c>
+      <c r="AD9" s="4">
+        <f>MAX(0,R9-MAX(0,X9-SUM(O9:Q9)))</f>
+        <v/>
+      </c>
+      <c r="AE9" s="4">
+        <f>MAX(0,S9-MAX(0,X9-SUM(O9:R9)))</f>
+        <v/>
+      </c>
+      <c r="AF9" s="4">
+        <f>MAX(0,T9-MAX(0,X9-SUM(O9:S9)))</f>
+        <v/>
+      </c>
+      <c r="AG9" s="4">
+        <f>MAX(0,U9-MAX(0,X9-SUM(O9:T9)))</f>
+        <v/>
+      </c>
+      <c r="AH9" s="4">
+        <f>MAX(0,V9-MAX(0,X9-SUM(O9:U9)))</f>
+        <v/>
+      </c>
+      <c r="AI9" s="4">
+        <f>MAX(0,W9-MAX(0,X9-SUM(O9:V9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802359</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>SWRG</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>202610072000</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>JPTYO</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx3 </t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>20260921</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>CY-RTN 21-23/09/26
+*PLS CHECK OPEN GATE BEFORE RETURN CTNR*</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="4">
+        <f>SUM(O10:W10)-X10</f>
+        <v/>
+      </c>
+      <c r="AA10" s="4">
+        <f>MAX(0,O10-MAX(0,X10))</f>
+        <v/>
+      </c>
+      <c r="AB10" s="4">
+        <f>MAX(0,P10-MAX(0,X10-SUM(O10:O10)))</f>
+        <v/>
+      </c>
+      <c r="AC10" s="4">
+        <f>MAX(0,Q10-MAX(0,X10-SUM(O10:P10)))</f>
+        <v/>
+      </c>
+      <c r="AD10" s="4">
+        <f>MAX(0,R10-MAX(0,X10-SUM(O10:Q10)))</f>
+        <v/>
+      </c>
+      <c r="AE10" s="4">
+        <f>MAX(0,S10-MAX(0,X10-SUM(O10:R10)))</f>
+        <v/>
+      </c>
+      <c r="AF10" s="4">
+        <f>MAX(0,T10-MAX(0,X10-SUM(O10:S10)))</f>
+        <v/>
+      </c>
+      <c r="AG10" s="4">
+        <f>MAX(0,U10-MAX(0,X10-SUM(O10:T10)))</f>
+        <v/>
+      </c>
+      <c r="AH10" s="4">
+        <f>MAX(0,V10-MAX(0,X10-SUM(O10:U10)))</f>
+        <v/>
+      </c>
+      <c r="AI10" s="4">
+        <f>MAX(0,W10-MAX(0,X10-SUM(O10:V10)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802360</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>SWRG</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>202610072000</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>JPTYO</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx4 </t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>20260921</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>CY-RTN 21-23/09/26
+*PLS CHECK OPEN GATE BEFORE RETURN CTNR*</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="4">
+        <f>SUM(O11:W11)-X11</f>
+        <v/>
+      </c>
+      <c r="AA11" s="4">
+        <f>MAX(0,O11-MAX(0,X11))</f>
+        <v/>
+      </c>
+      <c r="AB11" s="4">
+        <f>MAX(0,P11-MAX(0,X11-SUM(O11:O11)))</f>
+        <v/>
+      </c>
+      <c r="AC11" s="4">
+        <f>MAX(0,Q11-MAX(0,X11-SUM(O11:P11)))</f>
+        <v/>
+      </c>
+      <c r="AD11" s="4">
+        <f>MAX(0,R11-MAX(0,X11-SUM(O11:Q11)))</f>
+        <v/>
+      </c>
+      <c r="AE11" s="4">
+        <f>MAX(0,S11-MAX(0,X11-SUM(O11:R11)))</f>
+        <v/>
+      </c>
+      <c r="AF11" s="4">
+        <f>MAX(0,T11-MAX(0,X11-SUM(O11:S11)))</f>
+        <v/>
+      </c>
+      <c r="AG11" s="4">
+        <f>MAX(0,U11-MAX(0,X11-SUM(O11:T11)))</f>
+        <v/>
+      </c>
+      <c r="AH11" s="4">
+        <f>MAX(0,V11-MAX(0,X11-SUM(O11:U11)))</f>
+        <v/>
+      </c>
+      <c r="AI11" s="4">
+        <f>MAX(0,W11-MAX(0,X11-SUM(O11:V11)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802361</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>SWRG</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>202610072000</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>JPTYO</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx3 </t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>20260921</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>CY-RTN 21-23/09/26
+*PLS CHECK OPEN GATE BEFORE RETURN CTNR*</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="4">
+        <f>SUM(O12:W12)-X12</f>
+        <v/>
+      </c>
+      <c r="AA12" s="4">
+        <f>MAX(0,O12-MAX(0,X12))</f>
+        <v/>
+      </c>
+      <c r="AB12" s="4">
+        <f>MAX(0,P12-MAX(0,X12-SUM(O12:O12)))</f>
+        <v/>
+      </c>
+      <c r="AC12" s="4">
+        <f>MAX(0,Q12-MAX(0,X12-SUM(O12:P12)))</f>
+        <v/>
+      </c>
+      <c r="AD12" s="4">
+        <f>MAX(0,R12-MAX(0,X12-SUM(O12:Q12)))</f>
+        <v/>
+      </c>
+      <c r="AE12" s="4">
+        <f>MAX(0,S12-MAX(0,X12-SUM(O12:R12)))</f>
+        <v/>
+      </c>
+      <c r="AF12" s="4">
+        <f>MAX(0,T12-MAX(0,X12-SUM(O12:S12)))</f>
+        <v/>
+      </c>
+      <c r="AG12" s="4">
+        <f>MAX(0,U12-MAX(0,X12-SUM(O12:T12)))</f>
+        <v/>
+      </c>
+      <c r="AH12" s="4">
+        <f>MAX(0,V12-MAX(0,X12-SUM(O12:U12)))</f>
+        <v/>
+      </c>
+      <c r="AI12" s="4">
+        <f>MAX(0,W12-MAX(0,X12-SUM(O12:V12)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802484</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>SWMM</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>202609240000</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
           <t>JPIYM</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">20'x3 </t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>20260912</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>WHA GC LOGISTICS COMPANY LIMITED</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>RESIN</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">CY-RTN 12-15/09/26 (INV.3110001446) (1ST RTN DD: 18/09/26 WO/RENT)
 **CHECK OPENGATE BEFORE RETURN CNTR**
 </t>
         </is>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="O13" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="4">
-        <f>SUM(O4:W4)-X4</f>
-        <v/>
-      </c>
-      <c r="AA4" s="4">
-        <f>MAX(0,O4-MAX(0,X4))</f>
-        <v/>
-      </c>
-      <c r="AB4" s="4">
-        <f>MAX(0,P4-MAX(0,X4-SUM(O4:O4)))</f>
-        <v/>
-      </c>
-      <c r="AC4" s="4">
-        <f>MAX(0,Q4-MAX(0,X4-SUM(O4:P4)))</f>
-        <v/>
-      </c>
-      <c r="AD4" s="4">
-        <f>MAX(0,R4-MAX(0,X4-SUM(O4:Q4)))</f>
-        <v/>
-      </c>
-      <c r="AE4" s="4">
-        <f>MAX(0,S4-MAX(0,X4-SUM(O4:R4)))</f>
-        <v/>
-      </c>
-      <c r="AF4" s="4">
-        <f>MAX(0,T4-MAX(0,X4-SUM(O4:S4)))</f>
-        <v/>
-      </c>
-      <c r="AG4" s="4">
-        <f>MAX(0,U4-MAX(0,X4-SUM(O4:T4)))</f>
-        <v/>
-      </c>
-      <c r="AH4" s="4">
-        <f>MAX(0,V4-MAX(0,X4-SUM(O4:U4)))</f>
-        <v/>
-      </c>
-      <c r="AI4" s="4">
-        <f>MAX(0,W4-MAX(0,X4-SUM(O4:V4)))</f>
+      <c r="P13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z13" s="4">
+        <f>SUM(O13:W13)-X13</f>
+        <v/>
+      </c>
+      <c r="AA13" s="4">
+        <f>MAX(0,O13-MAX(0,X13))</f>
+        <v/>
+      </c>
+      <c r="AB13" s="4">
+        <f>MAX(0,P13-MAX(0,X13-SUM(O13:O13)))</f>
+        <v/>
+      </c>
+      <c r="AC13" s="4">
+        <f>MAX(0,Q13-MAX(0,X13-SUM(O13:P13)))</f>
+        <v/>
+      </c>
+      <c r="AD13" s="4">
+        <f>MAX(0,R13-MAX(0,X13-SUM(O13:Q13)))</f>
+        <v/>
+      </c>
+      <c r="AE13" s="4">
+        <f>MAX(0,S13-MAX(0,X13-SUM(O13:R13)))</f>
+        <v/>
+      </c>
+      <c r="AF13" s="4">
+        <f>MAX(0,T13-MAX(0,X13-SUM(O13:S13)))</f>
+        <v/>
+      </c>
+      <c r="AG13" s="4">
+        <f>MAX(0,U13-MAX(0,X13-SUM(O13:T13)))</f>
+        <v/>
+      </c>
+      <c r="AH13" s="4">
+        <f>MAX(0,V13-MAX(0,X13-SUM(O13:U13)))</f>
+        <v/>
+      </c>
+      <c r="AI13" s="4">
+        <f>MAX(0,W13-MAX(0,X13-SUM(O13:V13)))</f>
         <v/>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>HASLS22260802485</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>SWVG</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>2612N</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>202610030200</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>THLCH</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>JPIYM</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>20260909</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>WHA GC LOGISTICS COMPANY LIMITED</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>RESIN</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">CY-RTN 09-11/09/26 </t>
         </is>
       </c>
-      <c r="O5" s="4" t="n">
+      <c r="O14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="P5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="4">
-        <f>SUM(O5:W5)-X5</f>
-        <v/>
-      </c>
-      <c r="AA5" s="4">
-        <f>MAX(0,O5-MAX(0,X5))</f>
-        <v/>
-      </c>
-      <c r="AB5" s="4">
-        <f>MAX(0,P5-MAX(0,X5-SUM(O5:O5)))</f>
-        <v/>
-      </c>
-      <c r="AC5" s="4">
-        <f>MAX(0,Q5-MAX(0,X5-SUM(O5:P5)))</f>
-        <v/>
-      </c>
-      <c r="AD5" s="4">
-        <f>MAX(0,R5-MAX(0,X5-SUM(O5:Q5)))</f>
-        <v/>
-      </c>
-      <c r="AE5" s="4">
-        <f>MAX(0,S5-MAX(0,X5-SUM(O5:R5)))</f>
-        <v/>
-      </c>
-      <c r="AF5" s="4">
-        <f>MAX(0,T5-MAX(0,X5-SUM(O5:S5)))</f>
-        <v/>
-      </c>
-      <c r="AG5" s="4">
-        <f>MAX(0,U5-MAX(0,X5-SUM(O5:T5)))</f>
-        <v/>
-      </c>
-      <c r="AH5" s="4">
-        <f>MAX(0,V5-MAX(0,X5-SUM(O5:U5)))</f>
-        <v/>
-      </c>
-      <c r="AI5" s="4">
-        <f>MAX(0,W5-MAX(0,X5-SUM(O5:V5)))</f>
+      <c r="P14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z14" s="4">
+        <f>SUM(O14:W14)-X14</f>
+        <v/>
+      </c>
+      <c r="AA14" s="4">
+        <f>MAX(0,O14-MAX(0,X14))</f>
+        <v/>
+      </c>
+      <c r="AB14" s="4">
+        <f>MAX(0,P14-MAX(0,X14-SUM(O14:O14)))</f>
+        <v/>
+      </c>
+      <c r="AC14" s="4">
+        <f>MAX(0,Q14-MAX(0,X14-SUM(O14:P14)))</f>
+        <v/>
+      </c>
+      <c r="AD14" s="4">
+        <f>MAX(0,R14-MAX(0,X14-SUM(O14:Q14)))</f>
+        <v/>
+      </c>
+      <c r="AE14" s="4">
+        <f>MAX(0,S14-MAX(0,X14-SUM(O14:R14)))</f>
+        <v/>
+      </c>
+      <c r="AF14" s="4">
+        <f>MAX(0,T14-MAX(0,X14-SUM(O14:S14)))</f>
+        <v/>
+      </c>
+      <c r="AG14" s="4">
+        <f>MAX(0,U14-MAX(0,X14-SUM(O14:T14)))</f>
+        <v/>
+      </c>
+      <c r="AH14" s="4">
+        <f>MAX(0,V14-MAX(0,X14-SUM(O14:U14)))</f>
+        <v/>
+      </c>
+      <c r="AI14" s="4">
+        <f>MAX(0,W14-MAX(0,X14-SUM(O14:V14)))</f>
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802613</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>202610011100</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>HKHKG</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x7 </t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>CY-RTN 23-25/09/26
+*PLS CHECK OPEN GATE BEFORE RETURN CTNR*</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="4">
+        <f>SUM(O15:W15)-X15</f>
+        <v/>
+      </c>
+      <c r="AA15" s="4">
+        <f>MAX(0,O15-MAX(0,X15))</f>
+        <v/>
+      </c>
+      <c r="AB15" s="4">
+        <f>MAX(0,P15-MAX(0,X15-SUM(O15:O15)))</f>
+        <v/>
+      </c>
+      <c r="AC15" s="4">
+        <f>MAX(0,Q15-MAX(0,X15-SUM(O15:P15)))</f>
+        <v/>
+      </c>
+      <c r="AD15" s="4">
+        <f>MAX(0,R15-MAX(0,X15-SUM(O15:Q15)))</f>
+        <v/>
+      </c>
+      <c r="AE15" s="4">
+        <f>MAX(0,S15-MAX(0,X15-SUM(O15:R15)))</f>
+        <v/>
+      </c>
+      <c r="AF15" s="4">
+        <f>MAX(0,T15-MAX(0,X15-SUM(O15:S15)))</f>
+        <v/>
+      </c>
+      <c r="AG15" s="4">
+        <f>MAX(0,U15-MAX(0,X15-SUM(O15:T15)))</f>
+        <v/>
+      </c>
+      <c r="AH15" s="4">
+        <f>MAX(0,V15-MAX(0,X15-SUM(O15:U15)))</f>
+        <v/>
+      </c>
+      <c r="AI15" s="4">
+        <f>MAX(0,W15-MAX(0,X15-SUM(O15:V15)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260900120</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>SWSP</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>202610020330</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>KRPTK</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>20260928</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>SDS-ACUTECH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>3AC (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>AIR PURIFIER</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>Pickup : 2026-09-28, Return : 2026-09-28</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="4">
+        <f>SUM(O16:W16)-X16</f>
+        <v/>
+      </c>
+      <c r="AA16" s="4">
+        <f>MAX(0,O16-MAX(0,X16))</f>
+        <v/>
+      </c>
+      <c r="AB16" s="4">
+        <f>MAX(0,P16-MAX(0,X16-SUM(O16:O16)))</f>
+        <v/>
+      </c>
+      <c r="AC16" s="4">
+        <f>MAX(0,Q16-MAX(0,X16-SUM(O16:P16)))</f>
+        <v/>
+      </c>
+      <c r="AD16" s="4">
+        <f>MAX(0,R16-MAX(0,X16-SUM(O16:Q16)))</f>
+        <v/>
+      </c>
+      <c r="AE16" s="4">
+        <f>MAX(0,S16-MAX(0,X16-SUM(O16:R16)))</f>
+        <v/>
+      </c>
+      <c r="AF16" s="4">
+        <f>MAX(0,T16-MAX(0,X16-SUM(O16:S16)))</f>
+        <v/>
+      </c>
+      <c r="AG16" s="4">
+        <f>MAX(0,U16-MAX(0,X16-SUM(O16:T16)))</f>
+        <v/>
+      </c>
+      <c r="AH16" s="4">
+        <f>MAX(0,V16-MAX(0,X16-SUM(O16:U16)))</f>
+        <v/>
+      </c>
+      <c r="AI16" s="4">
+        <f>MAX(0,W16-MAX(0,X16-SUM(O16:V16)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5">
-        <f>SUM(O3:O5)</f>
-        <v/>
-      </c>
-      <c r="P6" s="5">
-        <f>SUM(P3:P5)</f>
-        <v/>
-      </c>
-      <c r="Q6" s="5">
-        <f>SUM(Q3:Q5)</f>
-        <v/>
-      </c>
-      <c r="R6" s="5">
-        <f>SUM(R3:R5)</f>
-        <v/>
-      </c>
-      <c r="S6" s="5">
-        <f>SUM(S3:S5)</f>
-        <v/>
-      </c>
-      <c r="T6" s="5">
-        <f>SUM(T3:T5)</f>
-        <v/>
-      </c>
-      <c r="U6" s="5">
-        <f>SUM(U3:U5)</f>
-        <v/>
-      </c>
-      <c r="V6" s="5">
-        <f>SUM(V3:V5)</f>
-        <v/>
-      </c>
-      <c r="W6" s="5">
-        <f>SUM(W3:W5)</f>
-        <v/>
-      </c>
-      <c r="X6" s="5">
-        <f>SUM(X3:X5)</f>
-        <v/>
-      </c>
-      <c r="Y6" s="5" t="n"/>
-      <c r="Z6" s="5">
-        <f>SUM(Z3:Z5)</f>
-        <v/>
-      </c>
-      <c r="AA6" s="5">
-        <f>SUM(AA3:AA5)</f>
-        <v/>
-      </c>
-      <c r="AB6" s="5">
-        <f>SUM(AB3:AB5)</f>
-        <v/>
-      </c>
-      <c r="AC6" s="5">
-        <f>SUM(AC3:AC5)</f>
-        <v/>
-      </c>
-      <c r="AD6" s="5">
-        <f>SUM(AD3:AD5)</f>
-        <v/>
-      </c>
-      <c r="AE6" s="5">
-        <f>SUM(AE3:AE5)</f>
-        <v/>
-      </c>
-      <c r="AF6" s="5">
-        <f>SUM(AF3:AF5)</f>
-        <v/>
-      </c>
-      <c r="AG6" s="5">
-        <f>SUM(AG3:AG5)</f>
-        <v/>
-      </c>
-      <c r="AH6" s="5">
-        <f>SUM(AH3:AH5)</f>
-        <v/>
-      </c>
-      <c r="AI6" s="5">
-        <f>SUM(AI3:AI5)</f>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="n"/>
+      <c r="K17" s="5" t="n"/>
+      <c r="L17" s="5" t="n"/>
+      <c r="M17" s="5" t="n"/>
+      <c r="N17" s="5" t="n"/>
+      <c r="O17" s="5">
+        <f>SUM(O3:O16)</f>
+        <v/>
+      </c>
+      <c r="P17" s="5">
+        <f>SUM(P3:P16)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="5">
+        <f>SUM(Q3:Q16)</f>
+        <v/>
+      </c>
+      <c r="R17" s="5">
+        <f>SUM(R3:R16)</f>
+        <v/>
+      </c>
+      <c r="S17" s="5">
+        <f>SUM(S3:S16)</f>
+        <v/>
+      </c>
+      <c r="T17" s="5">
+        <f>SUM(T3:T16)</f>
+        <v/>
+      </c>
+      <c r="U17" s="5">
+        <f>SUM(U3:U16)</f>
+        <v/>
+      </c>
+      <c r="V17" s="5">
+        <f>SUM(V3:V16)</f>
+        <v/>
+      </c>
+      <c r="W17" s="5">
+        <f>SUM(W3:W16)</f>
+        <v/>
+      </c>
+      <c r="X17" s="5">
+        <f>SUM(X3:X16)</f>
+        <v/>
+      </c>
+      <c r="Y17" s="5" t="n"/>
+      <c r="Z17" s="5">
+        <f>SUM(Z3:Z16)</f>
+        <v/>
+      </c>
+      <c r="AA17" s="5">
+        <f>SUM(AA3:AA16)</f>
+        <v/>
+      </c>
+      <c r="AB17" s="5">
+        <f>SUM(AB3:AB16)</f>
+        <v/>
+      </c>
+      <c r="AC17" s="5">
+        <f>SUM(AC3:AC16)</f>
+        <v/>
+      </c>
+      <c r="AD17" s="5">
+        <f>SUM(AD3:AD16)</f>
+        <v/>
+      </c>
+      <c r="AE17" s="5">
+        <f>SUM(AE3:AE16)</f>
+        <v/>
+      </c>
+      <c r="AF17" s="5">
+        <f>SUM(AF3:AF16)</f>
+        <v/>
+      </c>
+      <c r="AG17" s="5">
+        <f>SUM(AG3:AG16)</f>
+        <v/>
+      </c>
+      <c r="AH17" s="5">
+        <f>SUM(AH3:AH16)</f>
+        <v/>
+      </c>
+      <c r="AI17" s="5">
+        <f>SUM(AI3:AI16)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AI5"/>
+  <autoFilter ref="A2:AI16"/>
   <mergeCells count="1">
     <mergeCell ref="A1:AI1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Merge 9-15-BKGWK.xls into pending data; support multi-file merge
- build_booking_balance_report.py and build_dashboard.py now accept
  multiple source .xls files on the command line and merge their
  rows by BK No (later files override earlier ones on conflict),
  via a new merge_sources() helper. build_combined/build_per_pickup/
  full_name_map take headers/name_by_code directly instead of
  re-reading a single src_path, enabling this.
- Data update: merged the existing 9-14-PD pending set (104 BK No)
  with "9-15-BKGWK.xls" (458 rows, 457 new + 1 updated) -> 550 BK No
  outstanding, 1324 containers. Two depots reappear (UNITHAI
  CONTAINER TERMINAL, ICD LKT - Esco Ladkrabang GATE 2). One row
  still flagged for missing Pickup Name (HASLS22260900416).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AI$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AI$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI6"/>
+  <dimension ref="A1:AI8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -748,7 +748,7 @@
           <t>202609220700</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="inlineStr">
         <is>
           <t>THLCH</t>
@@ -872,22 +872,22 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802485</t>
+          <t>HASLS22260701913</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>202610031900</t>
+          <t>202609240200</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr"/>
@@ -898,52 +898,54 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20260918</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
+          <t>YUSEN LOGISTICS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>MAKITA MANUFACTURING (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t xml:space="preserve">ELECTRIC POWER TOOLS </t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>good, clean, dry, no leak, no hole, no smell, no oil container</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">CY-RTN 14-27/09/26 </t>
+          <t xml:space="preserve">Pickup : 2026-09-18, Return : 2026-09-20 (1ST RTN 20/09 W/O  RENT) 
+ ** PLEASE CHECK OPEN GATE BEFORE RETURN CNTR **
+</t>
         </is>
       </c>
       <c r="O4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>0</v>
@@ -1013,22 +1015,22 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260901089</t>
+          <t>HASLS22260802290</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>SWIC</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>202610031900</t>
+          <t>202609220500</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
@@ -1039,7 +1041,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>KRPUS</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1049,32 +1051,32 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
+          <t>ALUCON PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>ALUCON PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>EMPTY ALUMINIUM TUBES</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">CY-RTN 14-27/09/26 </t>
+          <t>Pickup : 2026-09-17, Return : 2026-09-19</t>
         </is>
       </c>
       <c r="O5" s="4" t="n">
@@ -1152,108 +1154,390 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802485</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>202610031900</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>JPIYM</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x2 </t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CY-RTN 14-27/09/26 </t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="4">
+        <f>SUM(O6:W6)-X6</f>
+        <v/>
+      </c>
+      <c r="AA6" s="4">
+        <f>MAX(0,O6-MAX(0,X6))</f>
+        <v/>
+      </c>
+      <c r="AB6" s="4">
+        <f>MAX(0,P6-MAX(0,X6-SUM(O6:O6)))</f>
+        <v/>
+      </c>
+      <c r="AC6" s="4">
+        <f>MAX(0,Q6-MAX(0,X6-SUM(O6:P6)))</f>
+        <v/>
+      </c>
+      <c r="AD6" s="4">
+        <f>MAX(0,R6-MAX(0,X6-SUM(O6:Q6)))</f>
+        <v/>
+      </c>
+      <c r="AE6" s="4">
+        <f>MAX(0,S6-MAX(0,X6-SUM(O6:R6)))</f>
+        <v/>
+      </c>
+      <c r="AF6" s="4">
+        <f>MAX(0,T6-MAX(0,X6-SUM(O6:S6)))</f>
+        <v/>
+      </c>
+      <c r="AG6" s="4">
+        <f>MAX(0,U6-MAX(0,X6-SUM(O6:T6)))</f>
+        <v/>
+      </c>
+      <c r="AH6" s="4">
+        <f>MAX(0,V6-MAX(0,X6-SUM(O6:U6)))</f>
+        <v/>
+      </c>
+      <c r="AI6" s="4">
+        <f>MAX(0,W6-MAX(0,X6-SUM(O6:V6)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260901089</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>202610031900</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>JPIYM</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CY-RTN 14-27/09/26 </t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="4">
+        <f>SUM(O7:W7)-X7</f>
+        <v/>
+      </c>
+      <c r="AA7" s="4">
+        <f>MAX(0,O7-MAX(0,X7))</f>
+        <v/>
+      </c>
+      <c r="AB7" s="4">
+        <f>MAX(0,P7-MAX(0,X7-SUM(O7:O7)))</f>
+        <v/>
+      </c>
+      <c r="AC7" s="4">
+        <f>MAX(0,Q7-MAX(0,X7-SUM(O7:P7)))</f>
+        <v/>
+      </c>
+      <c r="AD7" s="4">
+        <f>MAX(0,R7-MAX(0,X7-SUM(O7:Q7)))</f>
+        <v/>
+      </c>
+      <c r="AE7" s="4">
+        <f>MAX(0,S7-MAX(0,X7-SUM(O7:R7)))</f>
+        <v/>
+      </c>
+      <c r="AF7" s="4">
+        <f>MAX(0,T7-MAX(0,X7-SUM(O7:S7)))</f>
+        <v/>
+      </c>
+      <c r="AG7" s="4">
+        <f>MAX(0,U7-MAX(0,X7-SUM(O7:T7)))</f>
+        <v/>
+      </c>
+      <c r="AH7" s="4">
+        <f>MAX(0,V7-MAX(0,X7-SUM(O7:U7)))</f>
+        <v/>
+      </c>
+      <c r="AI7" s="4">
+        <f>MAX(0,W7-MAX(0,X7-SUM(O7:V7)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5">
-        <f>SUM(O3:O5)</f>
-        <v/>
-      </c>
-      <c r="P6" s="5">
-        <f>SUM(P3:P5)</f>
-        <v/>
-      </c>
-      <c r="Q6" s="5">
-        <f>SUM(Q3:Q5)</f>
-        <v/>
-      </c>
-      <c r="R6" s="5">
-        <f>SUM(R3:R5)</f>
-        <v/>
-      </c>
-      <c r="S6" s="5">
-        <f>SUM(S3:S5)</f>
-        <v/>
-      </c>
-      <c r="T6" s="5">
-        <f>SUM(T3:T5)</f>
-        <v/>
-      </c>
-      <c r="U6" s="5">
-        <f>SUM(U3:U5)</f>
-        <v/>
-      </c>
-      <c r="V6" s="5">
-        <f>SUM(V3:V5)</f>
-        <v/>
-      </c>
-      <c r="W6" s="5">
-        <f>SUM(W3:W5)</f>
-        <v/>
-      </c>
-      <c r="X6" s="5">
-        <f>SUM(X3:X5)</f>
-        <v/>
-      </c>
-      <c r="Y6" s="5" t="n"/>
-      <c r="Z6" s="5">
-        <f>SUM(Z3:Z5)</f>
-        <v/>
-      </c>
-      <c r="AA6" s="5">
-        <f>SUM(AA3:AA5)</f>
-        <v/>
-      </c>
-      <c r="AB6" s="5">
-        <f>SUM(AB3:AB5)</f>
-        <v/>
-      </c>
-      <c r="AC6" s="5">
-        <f>SUM(AC3:AC5)</f>
-        <v/>
-      </c>
-      <c r="AD6" s="5">
-        <f>SUM(AD3:AD5)</f>
-        <v/>
-      </c>
-      <c r="AE6" s="5">
-        <f>SUM(AE3:AE5)</f>
-        <v/>
-      </c>
-      <c r="AF6" s="5">
-        <f>SUM(AF3:AF5)</f>
-        <v/>
-      </c>
-      <c r="AG6" s="5">
-        <f>SUM(AG3:AG5)</f>
-        <v/>
-      </c>
-      <c r="AH6" s="5">
-        <f>SUM(AH3:AH5)</f>
-        <v/>
-      </c>
-      <c r="AI6" s="5">
-        <f>SUM(AI3:AI5)</f>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
+      <c r="L8" s="5" t="n"/>
+      <c r="M8" s="5" t="n"/>
+      <c r="N8" s="5" t="n"/>
+      <c r="O8" s="5">
+        <f>SUM(O3:O7)</f>
+        <v/>
+      </c>
+      <c r="P8" s="5">
+        <f>SUM(P3:P7)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="5">
+        <f>SUM(Q3:Q7)</f>
+        <v/>
+      </c>
+      <c r="R8" s="5">
+        <f>SUM(R3:R7)</f>
+        <v/>
+      </c>
+      <c r="S8" s="5">
+        <f>SUM(S3:S7)</f>
+        <v/>
+      </c>
+      <c r="T8" s="5">
+        <f>SUM(T3:T7)</f>
+        <v/>
+      </c>
+      <c r="U8" s="5">
+        <f>SUM(U3:U7)</f>
+        <v/>
+      </c>
+      <c r="V8" s="5">
+        <f>SUM(V3:V7)</f>
+        <v/>
+      </c>
+      <c r="W8" s="5">
+        <f>SUM(W3:W7)</f>
+        <v/>
+      </c>
+      <c r="X8" s="5">
+        <f>SUM(X3:X7)</f>
+        <v/>
+      </c>
+      <c r="Y8" s="5" t="n"/>
+      <c r="Z8" s="5">
+        <f>SUM(Z3:Z7)</f>
+        <v/>
+      </c>
+      <c r="AA8" s="5">
+        <f>SUM(AA3:AA7)</f>
+        <v/>
+      </c>
+      <c r="AB8" s="5">
+        <f>SUM(AB3:AB7)</f>
+        <v/>
+      </c>
+      <c r="AC8" s="5">
+        <f>SUM(AC3:AC7)</f>
+        <v/>
+      </c>
+      <c r="AD8" s="5">
+        <f>SUM(AD3:AD7)</f>
+        <v/>
+      </c>
+      <c r="AE8" s="5">
+        <f>SUM(AE3:AE7)</f>
+        <v/>
+      </c>
+      <c r="AF8" s="5">
+        <f>SUM(AF3:AF7)</f>
+        <v/>
+      </c>
+      <c r="AG8" s="5">
+        <f>SUM(AG3:AG7)</f>
+        <v/>
+      </c>
+      <c r="AH8" s="5">
+        <f>SUM(AH3:AH7)</f>
+        <v/>
+      </c>
+      <c r="AI8" s="5">
+        <f>SUM(AI3:AI7)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AI5"/>
+  <autoFilter ref="A2:AI7"/>
   <mergeCells count="1">
     <mergeCell ref="A1:AI1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Update dashboard and reports with 9-15-PD booking data
Regenerated from "9-15-PD.xls" (fresh full daily export, 2639
rows): 124 BK No outstanding, 287 containers — supersedes the
9-15-BKGWK merge from earlier today (this is the canonical daily
pending list). Removed the two per-depot files (UNITHAI CONTAINER
TERMINAL, ICD LKT - Esco Ladkrabang GATE 2) with no data in
today's list, and dropped the long-stale manual "Booking Balance
Summary - Copy.xlsx" artifact.

Note: HASLS22260900416 is still flagged for missing Pickup Name
(unresolved in the source system across the last three days' data).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AI$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AI$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI8"/>
+  <dimension ref="A1:AI6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -748,7 +748,7 @@
           <t>202609220700</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n"/>
+      <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="4" t="inlineStr">
         <is>
           <t>THLCH</t>
@@ -872,22 +872,22 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260701913</t>
+          <t>HASLS22260802485</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>SWMM</t>
+          <t>SWVG</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>202609240200</t>
+          <t>202610031830</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr"/>
@@ -898,54 +898,52 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>JPIYM</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>20260918</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>YUSEN LOGISTICS (THAILAND) CO., LTD.</t>
+          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>MAKITA MANUFACTURING (THAILAND) CO., LTD.</t>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ELECTRIC POWER TOOLS </t>
+          <t>RESIN</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>good, clean, dry, no leak, no hole, no smell, no oil container</t>
+          <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pickup : 2026-09-18, Return : 2026-09-20 (1ST RTN 20/09 W/O  RENT) 
- ** PLEASE CHECK OPEN GATE BEFORE RETURN CNTR **
-</t>
+          <t xml:space="preserve">CY-RTN 14-27/09/26 </t>
         </is>
       </c>
       <c r="O4" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>0</v>
@@ -1015,22 +1013,22 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802290</t>
+          <t>HASLS22260901089</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>SWVG</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>202609220500</t>
+          <t>202610031830</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
@@ -1041,7 +1039,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>KRPUS</t>
+          <t>JPIYM</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1051,32 +1049,32 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>20260917</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>ALUCON PUBLIC COMPANY LIMITED</t>
+          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>ALUCON PUBLIC COMPANY LIMITED</t>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>EMPTY ALUMINIUM TUBES</t>
+          <t>RESIN</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-17, Return : 2026-09-19</t>
+          <t xml:space="preserve">CY-RTN 14-27/09/26 </t>
         </is>
       </c>
       <c r="O5" s="4" t="n">
@@ -1154,390 +1152,108 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260802485</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>SWVG</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>202610031900</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>JPIYM</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x2 </t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>20260914</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>RESIN</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CTNR</t>
-        </is>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CY-RTN 14-27/09/26 </t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="4">
-        <f>SUM(O6:W6)-X6</f>
-        <v/>
-      </c>
-      <c r="AA6" s="4">
-        <f>MAX(0,O6-MAX(0,X6))</f>
-        <v/>
-      </c>
-      <c r="AB6" s="4">
-        <f>MAX(0,P6-MAX(0,X6-SUM(O6:O6)))</f>
-        <v/>
-      </c>
-      <c r="AC6" s="4">
-        <f>MAX(0,Q6-MAX(0,X6-SUM(O6:P6)))</f>
-        <v/>
-      </c>
-      <c r="AD6" s="4">
-        <f>MAX(0,R6-MAX(0,X6-SUM(O6:Q6)))</f>
-        <v/>
-      </c>
-      <c r="AE6" s="4">
-        <f>MAX(0,S6-MAX(0,X6-SUM(O6:R6)))</f>
-        <v/>
-      </c>
-      <c r="AF6" s="4">
-        <f>MAX(0,T6-MAX(0,X6-SUM(O6:S6)))</f>
-        <v/>
-      </c>
-      <c r="AG6" s="4">
-        <f>MAX(0,U6-MAX(0,X6-SUM(O6:T6)))</f>
-        <v/>
-      </c>
-      <c r="AH6" s="4">
-        <f>MAX(0,V6-MAX(0,X6-SUM(O6:U6)))</f>
-        <v/>
-      </c>
-      <c r="AI6" s="4">
-        <f>MAX(0,W6-MAX(0,X6-SUM(O6:V6)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260901089</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>SWVG</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>202610031900</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>JPIYM</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>20260914</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>WHA GC LOGISTICS COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>RESIN</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CTNR</t>
-        </is>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CY-RTN 14-27/09/26 </t>
-        </is>
-      </c>
-      <c r="O7" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="4">
-        <f>SUM(O7:W7)-X7</f>
-        <v/>
-      </c>
-      <c r="AA7" s="4">
-        <f>MAX(0,O7-MAX(0,X7))</f>
-        <v/>
-      </c>
-      <c r="AB7" s="4">
-        <f>MAX(0,P7-MAX(0,X7-SUM(O7:O7)))</f>
-        <v/>
-      </c>
-      <c r="AC7" s="4">
-        <f>MAX(0,Q7-MAX(0,X7-SUM(O7:P7)))</f>
-        <v/>
-      </c>
-      <c r="AD7" s="4">
-        <f>MAX(0,R7-MAX(0,X7-SUM(O7:Q7)))</f>
-        <v/>
-      </c>
-      <c r="AE7" s="4">
-        <f>MAX(0,S7-MAX(0,X7-SUM(O7:R7)))</f>
-        <v/>
-      </c>
-      <c r="AF7" s="4">
-        <f>MAX(0,T7-MAX(0,X7-SUM(O7:S7)))</f>
-        <v/>
-      </c>
-      <c r="AG7" s="4">
-        <f>MAX(0,U7-MAX(0,X7-SUM(O7:T7)))</f>
-        <v/>
-      </c>
-      <c r="AH7" s="4">
-        <f>MAX(0,V7-MAX(0,X7-SUM(O7:U7)))</f>
-        <v/>
-      </c>
-      <c r="AI7" s="4">
-        <f>MAX(0,W7-MAX(0,X7-SUM(O7:V7)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="5">
-        <f>SUM(O3:O7)</f>
-        <v/>
-      </c>
-      <c r="P8" s="5">
-        <f>SUM(P3:P7)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="5">
-        <f>SUM(Q3:Q7)</f>
-        <v/>
-      </c>
-      <c r="R8" s="5">
-        <f>SUM(R3:R7)</f>
-        <v/>
-      </c>
-      <c r="S8" s="5">
-        <f>SUM(S3:S7)</f>
-        <v/>
-      </c>
-      <c r="T8" s="5">
-        <f>SUM(T3:T7)</f>
-        <v/>
-      </c>
-      <c r="U8" s="5">
-        <f>SUM(U3:U7)</f>
-        <v/>
-      </c>
-      <c r="V8" s="5">
-        <f>SUM(V3:V7)</f>
-        <v/>
-      </c>
-      <c r="W8" s="5">
-        <f>SUM(W3:W7)</f>
-        <v/>
-      </c>
-      <c r="X8" s="5">
-        <f>SUM(X3:X7)</f>
-        <v/>
-      </c>
-      <c r="Y8" s="5" t="n"/>
-      <c r="Z8" s="5">
-        <f>SUM(Z3:Z7)</f>
-        <v/>
-      </c>
-      <c r="AA8" s="5">
-        <f>SUM(AA3:AA7)</f>
-        <v/>
-      </c>
-      <c r="AB8" s="5">
-        <f>SUM(AB3:AB7)</f>
-        <v/>
-      </c>
-      <c r="AC8" s="5">
-        <f>SUM(AC3:AC7)</f>
-        <v/>
-      </c>
-      <c r="AD8" s="5">
-        <f>SUM(AD3:AD7)</f>
-        <v/>
-      </c>
-      <c r="AE8" s="5">
-        <f>SUM(AE3:AE7)</f>
-        <v/>
-      </c>
-      <c r="AF8" s="5">
-        <f>SUM(AF3:AF7)</f>
-        <v/>
-      </c>
-      <c r="AG8" s="5">
-        <f>SUM(AG3:AG7)</f>
-        <v/>
-      </c>
-      <c r="AH8" s="5">
-        <f>SUM(AH3:AH7)</f>
-        <v/>
-      </c>
-      <c r="AI8" s="5">
-        <f>SUM(AI3:AI7)</f>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="5" t="n"/>
+      <c r="O6" s="5">
+        <f>SUM(O3:O5)</f>
+        <v/>
+      </c>
+      <c r="P6" s="5">
+        <f>SUM(P3:P5)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="5">
+        <f>SUM(Q3:Q5)</f>
+        <v/>
+      </c>
+      <c r="R6" s="5">
+        <f>SUM(R3:R5)</f>
+        <v/>
+      </c>
+      <c r="S6" s="5">
+        <f>SUM(S3:S5)</f>
+        <v/>
+      </c>
+      <c r="T6" s="5">
+        <f>SUM(T3:T5)</f>
+        <v/>
+      </c>
+      <c r="U6" s="5">
+        <f>SUM(U3:U5)</f>
+        <v/>
+      </c>
+      <c r="V6" s="5">
+        <f>SUM(V3:V5)</f>
+        <v/>
+      </c>
+      <c r="W6" s="5">
+        <f>SUM(W3:W5)</f>
+        <v/>
+      </c>
+      <c r="X6" s="5">
+        <f>SUM(X3:X5)</f>
+        <v/>
+      </c>
+      <c r="Y6" s="5" t="n"/>
+      <c r="Z6" s="5">
+        <f>SUM(Z3:Z5)</f>
+        <v/>
+      </c>
+      <c r="AA6" s="5">
+        <f>SUM(AA3:AA5)</f>
+        <v/>
+      </c>
+      <c r="AB6" s="5">
+        <f>SUM(AB3:AB5)</f>
+        <v/>
+      </c>
+      <c r="AC6" s="5">
+        <f>SUM(AC3:AC5)</f>
+        <v/>
+      </c>
+      <c r="AD6" s="5">
+        <f>SUM(AD3:AD5)</f>
+        <v/>
+      </c>
+      <c r="AE6" s="5">
+        <f>SUM(AE3:AE5)</f>
+        <v/>
+      </c>
+      <c r="AF6" s="5">
+        <f>SUM(AF3:AF5)</f>
+        <v/>
+      </c>
+      <c r="AG6" s="5">
+        <f>SUM(AG3:AG5)</f>
+        <v/>
+      </c>
+      <c r="AH6" s="5">
+        <f>SUM(AH3:AH5)</f>
+        <v/>
+      </c>
+      <c r="AI6" s="5">
+        <f>SUM(AI3:AI5)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AI7"/>
+  <autoFilter ref="A2:AI5"/>
   <mergeCells count="1">
     <mergeCell ref="A1:AI1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Drop raw booked-qty/Pickup/Return/Balance columns from per-pickup files
Removed GP22, GP42, GP45, RE22, RE45, UT22, UT42, PC22, PC42,
Pickup (qty), Return, and "Balance (Booked - Pickup)" from the
per-depot files — only the 9 "<Type> Remaining" net columns stay
(written as plain values now, since their source columns are no
longer on the sheet). TOTAL row sums those 9 columns. The
combined Booking Balance Summary.xlsx keeps all original columns
for audit purposes; this trim only applies to the simplified
per-pickup files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AG$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$U$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -103,27 +103,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -493,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG10"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -508,27 +499,15 @@
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="10" customWidth="1" min="23" max="23"/>
-    <col width="27" customWidth="1" min="24" max="24"/>
-    <col width="16" customWidth="1" min="25" max="25"/>
-    <col width="16" customWidth="1" min="26" max="26"/>
-    <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="16" customWidth="1" min="28" max="28"/>
-    <col width="16" customWidth="1" min="29" max="29"/>
-    <col width="16" customWidth="1" min="30" max="30"/>
-    <col width="16" customWidth="1" min="31" max="31"/>
-    <col width="16" customWidth="1" min="32" max="32"/>
-    <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1">
@@ -557,18 +536,6 @@
       <c r="S1" s="2" t="n"/>
       <c r="T1" s="2" t="n"/>
       <c r="U1" s="2" t="n"/>
-      <c r="V1" s="2" t="n"/>
-      <c r="W1" s="2" t="n"/>
-      <c r="X1" s="2" t="n"/>
-      <c r="Y1" s="2" t="n"/>
-      <c r="Z1" s="2" t="n"/>
-      <c r="AA1" s="2" t="n"/>
-      <c r="AB1" s="2" t="n"/>
-      <c r="AC1" s="2" t="n"/>
-      <c r="AD1" s="2" t="n"/>
-      <c r="AE1" s="2" t="n"/>
-      <c r="AF1" s="2" t="n"/>
-      <c r="AG1" s="2" t="n"/>
     </row>
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -631,520 +598,323 @@
           <t>TRAFFIC ORDER</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>GP22</t>
-        </is>
-      </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>GP42</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t>GP45</t>
-        </is>
-      </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>RE22</t>
-        </is>
-      </c>
-      <c r="Q2" s="4" t="inlineStr">
-        <is>
-          <t>RE45</t>
-        </is>
-      </c>
-      <c r="R2" s="4" t="inlineStr">
-        <is>
-          <t>UT22</t>
-        </is>
-      </c>
-      <c r="S2" s="4" t="inlineStr">
-        <is>
-          <t>UT42</t>
-        </is>
-      </c>
-      <c r="T2" s="4" t="inlineStr">
-        <is>
-          <t>PC22</t>
-        </is>
-      </c>
-      <c r="U2" s="4" t="inlineStr">
-        <is>
-          <t>PC42</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>Pickup</t>
-        </is>
-      </c>
-      <c r="W2" s="3" t="inlineStr">
-        <is>
-          <t>Return</t>
-        </is>
-      </c>
-      <c r="X2" s="3" t="inlineStr">
-        <is>
-          <t>Balance (Booked - Pickup)</t>
-        </is>
-      </c>
-      <c r="Y2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>GP22 Remaining</t>
         </is>
       </c>
-      <c r="Z2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>GP42 Remaining</t>
         </is>
       </c>
-      <c r="AA2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>GP45 Remaining</t>
         </is>
       </c>
-      <c r="AB2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>RE22 Remaining</t>
         </is>
       </c>
-      <c r="AC2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>RE45 Remaining</t>
         </is>
       </c>
-      <c r="AD2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>UT22 Remaining</t>
         </is>
       </c>
-      <c r="AE2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>UT42 Remaining</t>
         </is>
       </c>
-      <c r="AF2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>PC22 Remaining</t>
         </is>
       </c>
-      <c r="AG2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>PC42 Remaining</t>
         </is>
       </c>
     </row>
     <row r="3" ht="13" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>HASLS22260802485</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>SWVG</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>2612N</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>202610031800</t>
         </is>
       </c>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>THLCH</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>JPIYM</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>20260914</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>RESIN</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
-      <c r="M3" s="6" t="n">
+      <c r="M3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="N3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X3" s="5">
-        <f>SUM(M3:U3)-V3</f>
-        <v/>
-      </c>
-      <c r="Y3" s="5">
-        <f>MAX(0,M3-MAX(0,V3))</f>
-        <v/>
-      </c>
-      <c r="Z3" s="5">
-        <f>MAX(0,N3-MAX(0,V3-SUM(M3:M3)))</f>
-        <v/>
-      </c>
-      <c r="AA3" s="5">
-        <f>MAX(0,O3-MAX(0,V3-SUM(M3:N3)))</f>
-        <v/>
-      </c>
-      <c r="AB3" s="5">
-        <f>MAX(0,P3-MAX(0,V3-SUM(M3:O3)))</f>
-        <v/>
-      </c>
-      <c r="AC3" s="5">
-        <f>MAX(0,Q3-MAX(0,V3-SUM(M3:P3)))</f>
-        <v/>
-      </c>
-      <c r="AD3" s="5">
-        <f>MAX(0,R3-MAX(0,V3-SUM(M3:Q3)))</f>
-        <v/>
-      </c>
-      <c r="AE3" s="5">
-        <f>MAX(0,S3-MAX(0,V3-SUM(M3:R3)))</f>
-        <v/>
-      </c>
-      <c r="AF3" s="5">
-        <f>MAX(0,T3-MAX(0,V3-SUM(M3:S3)))</f>
-        <v/>
-      </c>
-      <c r="AG3" s="5">
-        <f>MAX(0,U3-MAX(0,V3-SUM(M3:T3)))</f>
-        <v/>
+      <c r="N3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4" ht="13" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>HASLS22260901089</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>SWVG</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>2612N</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>202610031800</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>THLCH</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>JPIYM</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>20260914</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>RESIN</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
-      <c r="M4" s="6" t="n">
+      <c r="M4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" s="5">
-        <f>SUM(M4:U4)-V4</f>
-        <v/>
-      </c>
-      <c r="Y4" s="5">
-        <f>MAX(0,M4-MAX(0,V4))</f>
-        <v/>
-      </c>
-      <c r="Z4" s="5">
-        <f>MAX(0,N4-MAX(0,V4-SUM(M4:M4)))</f>
-        <v/>
-      </c>
-      <c r="AA4" s="5">
-        <f>MAX(0,O4-MAX(0,V4-SUM(M4:N4)))</f>
-        <v/>
-      </c>
-      <c r="AB4" s="5">
-        <f>MAX(0,P4-MAX(0,V4-SUM(M4:O4)))</f>
-        <v/>
-      </c>
-      <c r="AC4" s="5">
-        <f>MAX(0,Q4-MAX(0,V4-SUM(M4:P4)))</f>
-        <v/>
-      </c>
-      <c r="AD4" s="5">
-        <f>MAX(0,R4-MAX(0,V4-SUM(M4:Q4)))</f>
-        <v/>
-      </c>
-      <c r="AE4" s="5">
-        <f>MAX(0,S4-MAX(0,V4-SUM(M4:R4)))</f>
-        <v/>
-      </c>
-      <c r="AF4" s="5">
-        <f>MAX(0,T4-MAX(0,V4-SUM(M4:S4)))</f>
-        <v/>
-      </c>
-      <c r="AG4" s="5">
-        <f>MAX(0,U4-MAX(0,V4-SUM(M4:T4)))</f>
-        <v/>
+      <c r="N4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5" ht="13" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-      <c r="M5" s="8">
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="5">
         <f>SUM(M3:M4)</f>
         <v/>
       </c>
-      <c r="N5" s="8">
+      <c r="N5" s="5">
         <f>SUM(N3:N4)</f>
         <v/>
       </c>
-      <c r="O5" s="8">
+      <c r="O5" s="5">
         <f>SUM(O3:O4)</f>
         <v/>
       </c>
-      <c r="P5" s="8">
+      <c r="P5" s="5">
         <f>SUM(P3:P4)</f>
         <v/>
       </c>
-      <c r="Q5" s="8">
+      <c r="Q5" s="5">
         <f>SUM(Q3:Q4)</f>
         <v/>
       </c>
-      <c r="R5" s="8">
+      <c r="R5" s="5">
         <f>SUM(R3:R4)</f>
         <v/>
       </c>
-      <c r="S5" s="8">
+      <c r="S5" s="5">
         <f>SUM(S3:S4)</f>
         <v/>
       </c>
-      <c r="T5" s="8">
+      <c r="T5" s="5">
         <f>SUM(T3:T4)</f>
         <v/>
       </c>
-      <c r="U5" s="8">
+      <c r="U5" s="5">
         <f>SUM(U3:U4)</f>
         <v/>
       </c>
-      <c r="V5" s="7">
-        <f>SUM(V3:V4)</f>
-        <v/>
-      </c>
-      <c r="W5" s="7" t="n"/>
-      <c r="X5" s="7">
-        <f>SUM(X3:X4)</f>
-        <v/>
-      </c>
-      <c r="Y5" s="7">
-        <f>SUM(Y3:Y4)</f>
-        <v/>
-      </c>
-      <c r="Z5" s="7">
-        <f>SUM(Z3:Z4)</f>
-        <v/>
-      </c>
-      <c r="AA5" s="7">
-        <f>SUM(AA3:AA4)</f>
-        <v/>
-      </c>
-      <c r="AB5" s="7">
-        <f>SUM(AB3:AB4)</f>
-        <v/>
-      </c>
-      <c r="AC5" s="7">
-        <f>SUM(AC3:AC4)</f>
-        <v/>
-      </c>
-      <c r="AD5" s="7">
-        <f>SUM(AD3:AD4)</f>
-        <v/>
-      </c>
-      <c r="AE5" s="7">
-        <f>SUM(AE3:AE4)</f>
-        <v/>
-      </c>
-      <c r="AF5" s="7">
-        <f>SUM(AF3:AF4)</f>
-        <v/>
-      </c>
-      <c r="AG5" s="7">
-        <f>SUM(AG3:AG4)</f>
-        <v/>
-      </c>
     </row>
     <row r="8" ht="13" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Pickup Name</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Number of Records</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Total Balance</t>
         </is>
       </c>
     </row>
     <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>CELLO</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="10" ht="13" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="5" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AG4"/>
+  <autoFilter ref="A2:U4"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:AG1"/>
+    <mergeCell ref="A1:U1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove title banner row from per-pickup files
Drops the "BKG PENDING (<codes>)" banner row entirely; the header
row now starts at row 1 and every subsequent row (data, TOTAL,
summary) shifts up by one accordingly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$U$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,19 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="13"/>
     </font>
     <font>
       <name val="Tahoma"/>
@@ -49,17 +43,12 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -103,20 +92,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -484,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U10"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -513,409 +500,379 @@
     <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BKG PENDING   (LCH28)</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="2" t="n"/>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="2" t="n"/>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="2" t="n"/>
-      <c r="S1" s="2" t="n"/>
-      <c r="T1" s="2" t="n"/>
-      <c r="U1" s="2" t="n"/>
+          <t>BK No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>VSL</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>VOY</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>POR</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>LOD</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>TPSZ</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>TRAN DT</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ORG CUST</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>COMMODITY</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>TRAFFIC ORDER</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>GP22</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>GP42</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>GP45</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>RE22</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>RE45</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>UT22</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>UT42</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>PC22</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>PC42</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="13" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>BK No</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>VSL</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>VOY</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>ETD</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>POR</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>LOD</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>DIS</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>TPSZ</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>TRAN DT</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>ORG CUST</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>COMMODITY</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>TRAFFIC ORDER</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>GP22</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>GP42</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>GP45</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>RE22</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>RE45</t>
-        </is>
-      </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>UT22</t>
-        </is>
-      </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>UT42</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>PC22</t>
-        </is>
-      </c>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>PC42</t>
-        </is>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802485</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>202610031800</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>JPIYM</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x2 </t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3" ht="13" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260802485</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260901089</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>SWVG</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>2612N</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>202610031800</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>THLCH</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>JPIYM</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x2 </t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>20260914</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>RESIN</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
-      <c r="M3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" s="4" t="n">
+      <c r="M3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" ht="13" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260901089</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>SWVG</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>202610031800</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>JPIYM</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>20260914</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>RESIN</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CTNR</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>0</v>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3">
+        <f>SUM(M2:M3)</f>
+        <v/>
+      </c>
+      <c r="N4" s="3">
+        <f>SUM(N2:N3)</f>
+        <v/>
+      </c>
+      <c r="O4" s="3">
+        <f>SUM(O2:O3)</f>
+        <v/>
+      </c>
+      <c r="P4" s="3">
+        <f>SUM(P2:P3)</f>
+        <v/>
+      </c>
+      <c r="Q4" s="3">
+        <f>SUM(Q2:Q3)</f>
+        <v/>
+      </c>
+      <c r="R4" s="3">
+        <f>SUM(R2:R3)</f>
+        <v/>
+      </c>
+      <c r="S4" s="3">
+        <f>SUM(S2:S3)</f>
+        <v/>
+      </c>
+      <c r="T4" s="3">
+        <f>SUM(T2:T3)</f>
+        <v/>
+      </c>
+      <c r="U4" s="3">
+        <f>SUM(U2:U3)</f>
+        <v/>
       </c>
     </row>
-    <row r="5" ht="13" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5">
-        <f>SUM(M3:M4)</f>
-        <v/>
-      </c>
-      <c r="N5" s="5">
-        <f>SUM(N3:N4)</f>
-        <v/>
-      </c>
-      <c r="O5" s="5">
-        <f>SUM(O3:O4)</f>
-        <v/>
-      </c>
-      <c r="P5" s="5">
-        <f>SUM(P3:P4)</f>
-        <v/>
-      </c>
-      <c r="Q5" s="5">
-        <f>SUM(Q3:Q4)</f>
-        <v/>
-      </c>
-      <c r="R5" s="5">
-        <f>SUM(R3:R4)</f>
-        <v/>
-      </c>
-      <c r="S5" s="5">
-        <f>SUM(S3:S4)</f>
-        <v/>
-      </c>
-      <c r="T5" s="5">
-        <f>SUM(T3:T4)</f>
-        <v/>
-      </c>
-      <c r="U5" s="5">
-        <f>SUM(U3:U4)</f>
-        <v/>
+    <row r="7" ht="13" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
       </c>
     </row>
     <row r="8" ht="13" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>สรุปยอดบุ๊คทั้งหมด</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" ht="13" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>สรุปยอดบุ๊คทั้งหมด</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C10" s="5" t="n">
+      <c r="C9" s="3" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:U4"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:U1"/>
-  </mergeCells>
+  <autoFilter ref="A1:U3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Replace pending data with 9-21-BKG-3WK.xls (3-week booking window)
Per user confirmation, this replaces the prior 9-17-PD snapshot
entirely and is used as today's pending list: 955 BK No
outstanding (2,385 containers) across 9 depots, including three
new ones (ICD LKT - Esco Ladkrabang GATE 2, UNITHAI CONTAINER
TERMINAL, YJC DEPOT). No rows flagged for missing Pickup Name
this run. Source is a forward-looking 3-week booking export
rather than the usual full daily PD list, hence the much larger
outstanding count than 9-17's 125.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,7 @@
     <col width="4" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
@@ -607,22 +607,22 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802485</t>
+          <t>HASLS22260801507</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610031800</t>
+          <t>202610200600</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -633,42 +633,43 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>KRPTK</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">40Hx40 </t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20261010</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>REFRIGERATOR</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>*No containers with cut and patch marks inside*
+GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>0</v>
@@ -692,22 +693,22 @@
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901089</t>
+          <t>HASLS22260802124</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>DJCF</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>0152N</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>202610031800</t>
+          <t>202610111600</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -718,42 +719,43 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>KRPTK</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx8 </t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20261002</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>WASHING MATCHINE</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>*No containers with cut and patch marks inside*
+GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P3" s="2" t="n">
         <v>0</v>
@@ -775,104 +777,1040 @@
       </c>
     </row>
     <row r="4" ht="13" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3">
-        <f>SUM(M2:M3)</f>
-        <v/>
-      </c>
-      <c r="N4" s="3">
-        <f>SUM(N2:N3)</f>
-        <v/>
-      </c>
-      <c r="O4" s="3">
-        <f>SUM(O2:O3)</f>
-        <v/>
-      </c>
-      <c r="P4" s="3">
-        <f>SUM(P2:P3)</f>
-        <v/>
-      </c>
-      <c r="Q4" s="3">
-        <f>SUM(Q2:Q3)</f>
-        <v/>
-      </c>
-      <c r="R4" s="3">
-        <f>SUM(R2:R3)</f>
-        <v/>
-      </c>
-      <c r="S4" s="3">
-        <f>SUM(S2:S3)</f>
-        <v/>
-      </c>
-      <c r="T4" s="3">
-        <f>SUM(T2:T3)</f>
-        <v/>
-      </c>
-      <c r="U4" s="3">
-        <f>SUM(U2:U3)</f>
-        <v/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802276</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>202610051300</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>TWKEL</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>20260924</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>L. LIGHTING GLASS CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>GLASS TUBES FOR ELECTRIC LIGHTING</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="13" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802359</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>SWRG</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>202610100330</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>JPTYO</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx3 </t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="13" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802360</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>202610061700</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>JPMYJ</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx5 </t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="13" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802361</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>SWRG</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>202610100330</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>JPTYO</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx3 </t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="2" t="n">
+          <t>HASLS22260802484</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>SWSP</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>202610060400</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>JPTKY</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x3 </t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
         <v>3</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802485</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>202610061700</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>JPIYM</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x2 </t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="13" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802613</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>202610051300</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>HKHKG</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x4 </t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="13" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260900119</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>DJCF</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>0152N</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>202610111600</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>KRPTK</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>20261006</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>3AC (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>AIR PURIFIER</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="13" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260900120</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SWSP</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>202610060400</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>KRPTK</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>20260928</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>3AC (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>AIR PURIFIER</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="13" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260901089</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>202610061700</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>JPIYM</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="13" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260901745</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DJCF</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>0152N</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>202610111600</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>KRPTK</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx8 </t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>20261002</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>WASHING MATCHINE</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>*No containers with cut and patch marks inside*
+GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="13" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3">
+        <f>SUM(M2:M14)</f>
+        <v/>
+      </c>
+      <c r="N15" s="3">
+        <f>SUM(N2:N14)</f>
+        <v/>
+      </c>
+      <c r="O15" s="3">
+        <f>SUM(O2:O14)</f>
+        <v/>
+      </c>
+      <c r="P15" s="3">
+        <f>SUM(P2:P14)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="3">
+        <f>SUM(Q2:Q14)</f>
+        <v/>
+      </c>
+      <c r="R15" s="3">
+        <f>SUM(R2:R14)</f>
+        <v/>
+      </c>
+      <c r="S15" s="3">
+        <f>SUM(S2:S14)</f>
+        <v/>
+      </c>
+      <c r="T15" s="3">
+        <f>SUM(T2:T14)</f>
+        <v/>
+      </c>
+      <c r="U15" s="3">
+        <f>SUM(U2:U14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="13" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="13" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" ht="13" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>3</v>
+      <c r="B20" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U3"/>
+  <autoFilter ref="A1:U14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update dashboard and reports with 9-24-PD+BKG-3WK data
Regenerated from "9-24-PD+BKG-3WK.xls" (970 rows, single clean
sheet): 970 BK No outstanding (2,434 containers) across 8 depots,
including ICD LKT and UNITHAI CONTAINER TERMINAL again. No rows
flagged for missing Pickup Name. Filename indicates this combines
the daily PD list and the 3-week booking window in one export.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,7 @@
     <col width="4" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
@@ -607,22 +607,22 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802485</t>
+          <t>HASLS22260801507</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610061700</t>
+          <t>202610190700</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -633,42 +633,43 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>KRPTK</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">40Hx40 </t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20261010</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>REFRIGERATOR</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>*No containers with cut and patch marks inside*
+GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>0</v>
@@ -692,22 +693,22 @@
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901089</t>
+          <t>HASLS22260802124</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>DJCF</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>0152N</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>202610061700</t>
+          <t>202610111800</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -718,42 +719,43 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>KRPTK</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx8 </t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20261002</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>WASHING MATCHINE</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>*No containers with cut and patch marks inside*
+GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P3" s="2" t="n">
         <v>0</v>
@@ -775,104 +777,1040 @@
       </c>
     </row>
     <row r="4" ht="13" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3">
-        <f>SUM(M2:M3)</f>
-        <v/>
-      </c>
-      <c r="N4" s="3">
-        <f>SUM(N2:N3)</f>
-        <v/>
-      </c>
-      <c r="O4" s="3">
-        <f>SUM(O2:O3)</f>
-        <v/>
-      </c>
-      <c r="P4" s="3">
-        <f>SUM(P2:P3)</f>
-        <v/>
-      </c>
-      <c r="Q4" s="3">
-        <f>SUM(Q2:Q3)</f>
-        <v/>
-      </c>
-      <c r="R4" s="3">
-        <f>SUM(R2:R3)</f>
-        <v/>
-      </c>
-      <c r="S4" s="3">
-        <f>SUM(S2:S3)</f>
-        <v/>
-      </c>
-      <c r="T4" s="3">
-        <f>SUM(T2:T3)</f>
-        <v/>
-      </c>
-      <c r="U4" s="3">
-        <f>SUM(U2:U3)</f>
-        <v/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802276</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>202610071200</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>TWKEL</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>20260924</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>L. LIGHTING GLASS CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>GLASS TUBES FOR ELECTRIC LIGHTING</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="13" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802359</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>SWRG</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>202610102230</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>JPTYO</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx3 </t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="13" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802360</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>202610080200</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>JPMYJ</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx5 </t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="13" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802361</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>SWRG</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>202610102230</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>JPTYO</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx3 </t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>3</v>
+          <t>HASLS22260802484</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>SWSP</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>202610060400</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>JPTKY</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x3 </t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802485</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>202610080200</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>JPIYM</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x2 </t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="13" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260802613</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>202610071200</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>HKHKG</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x4 </t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="13" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260900119</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>DJCF</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>0152N</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>202610111800</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>KRPTK</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>20261006</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>3AC (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>AIR PURIFIER</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="13" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260900120</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SWSP</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>202610060400</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>KRPTK</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>20260928</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>3AC (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>AIR PURIFIER</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="13" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260901089</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>202610080200</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>JPIYM</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="13" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260901745</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DJCF</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>0152N</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>202610111800</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>KRPTK</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx8 </t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>20261002</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>WASHING MATCHINE</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>*No containers with cut and patch marks inside*
+GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="13" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3">
+        <f>SUM(M2:M14)</f>
+        <v/>
+      </c>
+      <c r="N15" s="3">
+        <f>SUM(N2:N14)</f>
+        <v/>
+      </c>
+      <c r="O15" s="3">
+        <f>SUM(O2:O14)</f>
+        <v/>
+      </c>
+      <c r="P15" s="3">
+        <f>SUM(P2:P14)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="3">
+        <f>SUM(Q2:Q14)</f>
+        <v/>
+      </c>
+      <c r="R15" s="3">
+        <f>SUM(R2:R14)</f>
+        <v/>
+      </c>
+      <c r="S15" s="3">
+        <f>SUM(S2:S14)</f>
+        <v/>
+      </c>
+      <c r="T15" s="3">
+        <f>SUM(T2:T14)</f>
+        <v/>
+      </c>
+      <c r="U15" s="3">
+        <f>SUM(U2:U14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="13" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="13" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" ht="13" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>3</v>
+      <c r="B20" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U3"/>
+  <autoFilter ref="A1:U14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update dashboard and reports with 9-25-PD+BKG-3WK data
Regenerated from "9-25-PD+BKG-3WK.xls" (951 rows, single clean
sheet): 939 BK No outstanding (2,339 containers) across the same
8 depots as yesterday. No rows flagged for missing Pickup Name.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U20"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -622,7 +622,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610190700</t>
+          <t>202610191000</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -693,22 +693,22 @@
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802124</t>
+          <t>HASLS22260801555</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DJCF</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>0152N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>202610111800</t>
+          <t>202610040500</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -719,33 +719,32 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>KRPTK</t>
+          <t>JPSDJ</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx8 </t>
+          <t xml:space="preserve">40Hx3 </t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>20261002</t>
+          <t>20260928</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
+          <t>OSC SIAM SILICA CO., LTD.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>WASHING MATCHINE</t>
+          <t>SILICON DIOXIDE</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>*No containers with cut and patch marks inside*
-GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
@@ -755,7 +754,7 @@
         <v>0</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="P3" s="2" t="n">
         <v>0</v>
@@ -815,7 +814,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>20260924</t>
+          <t>20261003</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -864,7 +863,7 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802359</t>
+          <t>HASLS22260802361</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -949,22 +948,22 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802360</t>
+          <t>HASLS22260802485</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>HMVY</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>202610080200</t>
+          <t>202610180230</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -975,17 +974,17 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>JPMYJ</t>
+          <t>JPIYM</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx5 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>20260923</t>
+          <t>20261007</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1004,13 +1003,13 @@
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P6" s="2" t="n">
         <v>0</v>
@@ -1034,22 +1033,22 @@
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802361</t>
+          <t>HASLS22260900119</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>SWRG</t>
+          <t>DJCF</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>0152N</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>202610102230</t>
+          <t>202610111800</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -1060,32 +1059,32 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>JPTYO</t>
+          <t>KRPTK</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx3 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>20260923</t>
+          <t>20261006</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>3AC (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>AIR PURIFIER</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M7" s="2" t="n">
@@ -1095,7 +1094,7 @@
         <v>0</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P7" s="2" t="n">
         <v>0</v>
@@ -1119,12 +1118,12 @@
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802484</t>
+          <t>HASLS22260900647</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SWSP</t>
+          <t>SWRG</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1134,7 +1133,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>202610060400</t>
+          <t>202610112230</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -1145,42 +1144,42 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>JPTKY</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x3 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>20260923</t>
+          <t>20260928</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>GROHE SIAM LIMITED</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>SANITARY WARE</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>Request dry, Strong floor and good container condition</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P8" s="2" t="n">
         <v>0</v>
@@ -1204,22 +1203,22 @@
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802485</t>
+          <t>HASLS22260901089</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>KUS</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2616N</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>202610080200</t>
+          <t>202610140000</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -1235,12 +1234,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20261005</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1259,7 +1258,7 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -1289,22 +1288,22 @@
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802613</t>
+          <t>HASLS22260901355</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>SWAT</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>202610071200</t>
+          <t>202610040500</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -1315,42 +1314,42 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x4 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>20260923</t>
+          <t>20260928</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>HMC POLYMERS CO., LTD.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>POLYPROPYLENE</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P10" s="2" t="n">
         <v>0</v>
@@ -1374,22 +1373,22 @@
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900119</t>
+          <t>HASLS22260901914</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>DJCF</t>
+          <t>SWVG</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>0152N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>202610111800</t>
+          <t>202610080200</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
@@ -1400,32 +1399,32 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>KRPTK</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>20261006</t>
+          <t>20260928</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>3AC (THAILAND) CO., LTD.</t>
+          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>AIR PURIFIER</t>
+          <t>SILICONE</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>Good , Clean, No smell container are requested.</t>
         </is>
       </c>
       <c r="M11" s="2" t="n">
@@ -1435,7 +1434,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P11" s="2" t="n">
         <v>0</v>
@@ -1459,22 +1458,22 @@
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900120</t>
+          <t>HASLS22260901915</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SWSP</t>
+          <t>SWVG</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>202610060400</t>
+          <t>202610080200</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -1485,7 +1484,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>KRPTK</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1500,17 +1499,17 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>3AC (THAILAND) CO., LTD.</t>
+          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>AIR PURIFIER</t>
+          <t>SILICONE</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>Good , Clean, No smell container are requested.</t>
         </is>
       </c>
       <c r="M12" s="2" t="n">
@@ -1542,275 +1541,104 @@
       </c>
     </row>
     <row r="13" ht="13" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260901089</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>SWVG</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>202610080200</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>JPIYM</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>20260914</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>RESIN</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CTNR</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" s="2" t="n">
-        <v>0</v>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3">
+        <f>SUM(M2:M12)</f>
+        <v/>
+      </c>
+      <c r="N13" s="3">
+        <f>SUM(N2:N12)</f>
+        <v/>
+      </c>
+      <c r="O13" s="3">
+        <f>SUM(O2:O12)</f>
+        <v/>
+      </c>
+      <c r="P13" s="3">
+        <f>SUM(P2:P12)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="3">
+        <f>SUM(Q2:Q12)</f>
+        <v/>
+      </c>
+      <c r="R13" s="3">
+        <f>SUM(R2:R12)</f>
+        <v/>
+      </c>
+      <c r="S13" s="3">
+        <f>SUM(S2:S12)</f>
+        <v/>
+      </c>
+      <c r="T13" s="3">
+        <f>SUM(T2:T12)</f>
+        <v/>
+      </c>
+      <c r="U13" s="3">
+        <f>SUM(U2:U12)</f>
+        <v/>
       </c>
     </row>
-    <row r="14" ht="13" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260901745</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>DJCF</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>0152N</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>202610111800</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>KRPTK</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40Hx8 </t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>20261002</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>WASHING MATCHINE</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>*No containers with cut and patch marks inside*
-GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="P14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U14" s="2" t="n">
-        <v>0</v>
+    <row r="16" ht="13" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
       </c>
     </row>
-    <row r="15" ht="13" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="3">
-        <f>SUM(M2:M14)</f>
-        <v/>
-      </c>
-      <c r="N15" s="3">
-        <f>SUM(N2:N14)</f>
-        <v/>
-      </c>
-      <c r="O15" s="3">
-        <f>SUM(O2:O14)</f>
-        <v/>
-      </c>
-      <c r="P15" s="3">
-        <f>SUM(P2:P14)</f>
-        <v/>
-      </c>
-      <c r="Q15" s="3">
-        <f>SUM(Q2:Q14)</f>
-        <v/>
-      </c>
-      <c r="R15" s="3">
-        <f>SUM(R2:R14)</f>
-        <v/>
-      </c>
-      <c r="S15" s="3">
-        <f>SUM(S2:S14)</f>
-        <v/>
-      </c>
-      <c r="T15" s="3">
-        <f>SUM(T2:T14)</f>
-        <v/>
-      </c>
-      <c r="U15" s="3">
-        <f>SUM(U2:U14)</f>
-        <v/>
+    <row r="17" ht="13" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>56</v>
       </c>
     </row>
     <row r="18" ht="13" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="13" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="20" ht="13" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="C20" s="3" t="n">
-        <v>78</v>
+      <c r="B18" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U14"/>
+  <autoFilter ref="A1:U12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update dashboard and reports, merging 9-29-PENDING + 9-29-BKG-3WK
Two separate source files this time, merged by BK No (BKG-3WK
overrides PENDING on the 1 overlapping BK No): 134 + 904 new =
1,038 BK No outstanding, 2,691 containers, across the same 8
depots as recent days. No rows flagged for missing Pickup Name.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,7 @@
     <col width="4" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
@@ -607,12 +607,12 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260801507</t>
+          <t>HASLS22260802276</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SWMM</t>
+          <t>SWAT</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610191000</t>
+          <t>202610081000</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -633,43 +633,42 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>KRPTK</t>
+          <t>TWKEL</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx40 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>20261010</t>
+          <t>20261003</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>THAI SAMSUNG ELECTRONICS CO., LTD.</t>
+          <t>L. LIGHTING GLASS CO., LTD.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>REFRIGERATOR</t>
+          <t>GLASS TUBES FOR ELECTRIC LIGHTING</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>*No containers with cut and patch marks inside*
-GOOD CLEAN CONTIANER NO BLEAM (ELECTRONICS GOODS)</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>0</v>
@@ -693,22 +692,22 @@
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260801555</t>
+          <t>HASLS22260802361</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>KMBK</t>
+          <t>SWRG</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>202610040500</t>
+          <t>202610131130</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -719,7 +718,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>JPSDJ</t>
+          <t>JPTYO</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -729,22 +728,22 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>20260928</t>
+          <t>20260923</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>OSC SIAM SILICA CO., LTD.</t>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>SILICON DIOXIDE</t>
+          <t>RESIN</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
@@ -778,22 +777,22 @@
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802276</t>
+          <t>HASLS22260802485</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SWAT</t>
+          <t>HMVY</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>202610071200</t>
+          <t>202610200330</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -804,36 +803,36 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>TWKEL</t>
+          <t>JPIYM</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>20261003</t>
+          <t>20261007</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>L. LIGHTING GLASS CO., LTD.</t>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>GLASS TUBES FOR ELECTRIC LIGHTING</t>
+          <t>RESIN</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -863,7 +862,7 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802361</t>
+          <t>HASLS22260900838</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -878,7 +877,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>202610102230</t>
+          <t>202610131130</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -889,22 +888,22 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>JPTYO</t>
+          <t>JPNAH</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx3 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>20260923</t>
+          <t>20260930</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>THAI POLYETHYLENE CO., LTD.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -914,17 +913,17 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>RESIN-PALLET,NO RED WALL CONTAINER,CLEAN CONTAINER NO OIL STAINS , NO RUSTY ,NO CUT OR HOLE</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P5" s="2" t="n">
         <v>0</v>
@@ -948,22 +947,22 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802485</t>
+          <t>HASLS22260900975</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>HMVY</t>
+          <t>KMSU</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>202610180230</t>
+          <t>202610251730</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -974,7 +973,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -984,22 +983,22 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>20261007</t>
+          <t>20260930</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>TANATEX CHEMICALS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>CHEMICALS PRODUCT (NON DG)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
@@ -1033,22 +1032,22 @@
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900119</t>
+          <t>HASLS22260901089</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>DJCF</t>
+          <t>KUS</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>0152N</t>
+          <t>2616N</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>202610111800</t>
+          <t>202610150400</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -1059,42 +1058,42 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>KRPTK</t>
+          <t>JPIYM</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>20261006</t>
+          <t>20261005</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>3AC (THAILAND) CO., LTD.</t>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>AIR PURIFIER</t>
+          <t>RESIN</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P7" s="2" t="n">
         <v>0</v>
@@ -1118,22 +1117,22 @@
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900647</t>
+          <t>HASLS22260901355</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SWRG</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>202610112230</t>
+          <t>202610040100</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -1144,7 +1143,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1159,17 +1158,17 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>GROHE SIAM LIMITED</t>
+          <t>HMC POLYMERS CO., LTD.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>SANITARY WARE</t>
+          <t>POLYPROPYLENE</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Request dry, Strong floor and good container condition</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
@@ -1203,22 +1202,22 @@
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901089</t>
+          <t>HASLS22260901356</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>KUS</t>
+          <t>KXM</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2616N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>202610140000</t>
+          <t>202610100500</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -1229,42 +1228,42 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx4 </t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>20261005</t>
+          <t>20261001</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>THAI-YAZAKI ELECTRIC WIRE CO.,LTD.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>COPPER WIRE ROD</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>REQUEST CONTAINER GRADE A</t>
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P9" s="2" t="n">
         <v>0</v>
@@ -1288,7 +1287,7 @@
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901355</t>
+          <t>HASLS22260901548</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1303,7 +1302,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>202610040500</t>
+          <t>202610040100</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -1314,7 +1313,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>KRKAN</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1324,17 +1323,17 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>20260928</t>
+          <t>20261001</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>HMC POLYMERS CO., LTD.</t>
+          <t>Y-MECO CO., LTD.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>POLYPROPYLENE</t>
+          <t>ASSY COND</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1373,7 +1372,7 @@
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901914</t>
+          <t>HASLS22260901686</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1388,7 +1387,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>202610080200</t>
+          <t>202610070330</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
@@ -1399,42 +1398,42 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>JPNGO</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>20260928</t>
+          <t>20260930</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
+          <t>TANATEX CHEMICALS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>SILICONE</t>
+          <t>CHEMICALS PRODUCT DG CARGO</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Good , Clean, No smell container are requested.</t>
+          <t>**APPROVAL DG IN SYSTEM DD.24/09/2026** MIX DG22GPx1 (CLS 9 / UN 3082, CLS 8 / UN 3265)</t>
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P11" s="2" t="n">
         <v>0</v>
@@ -1458,22 +1457,22 @@
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901915</t>
+          <t>HASLS22260901795</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>202610080200</t>
+          <t>202610040100</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -1484,7 +1483,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1494,22 +1493,22 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>20260928</t>
+          <t>20260930</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
+          <t>TRI-WALL PACKAGING (THAI) LTD.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>SILICONE</t>
+          <t>CORRUGATED PAPER BOARD</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Good , Clean, No smell container are requested.</t>
+          <t>RQS CLEAN &amp; GOOD CONTAINER CONDITION.</t>
         </is>
       </c>
       <c r="M12" s="2" t="n">
@@ -1541,104 +1540,869 @@
       </c>
     </row>
     <row r="13" ht="13" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3">
-        <f>SUM(M2:M12)</f>
-        <v/>
-      </c>
-      <c r="N13" s="3">
-        <f>SUM(N2:N12)</f>
-        <v/>
-      </c>
-      <c r="O13" s="3">
-        <f>SUM(O2:O12)</f>
-        <v/>
-      </c>
-      <c r="P13" s="3">
-        <f>SUM(P2:P12)</f>
-        <v/>
-      </c>
-      <c r="Q13" s="3">
-        <f>SUM(Q2:Q12)</f>
-        <v/>
-      </c>
-      <c r="R13" s="3">
-        <f>SUM(R2:R12)</f>
-        <v/>
-      </c>
-      <c r="S13" s="3">
-        <f>SUM(S2:S12)</f>
-        <v/>
-      </c>
-      <c r="T13" s="3">
-        <f>SUM(T2:T12)</f>
-        <v/>
-      </c>
-      <c r="U13" s="3">
-        <f>SUM(U2:U12)</f>
-        <v/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260901914</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>202610070330</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>CNSHA</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx2 </t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>20260928</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>SILICONE</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Good , Clean, No smell container are requested.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="13" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260901915</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>202610070330</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>CNSHA</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>20260928</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>SILICONE</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Good , Clean, No smell container are requested.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="13" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260901971</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>202610040100</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x2 </t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>20260930</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>BANGKOK CRYSTAL CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>GLASS BLOCK</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="13" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902009</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>202610040100</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>KRPUS</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>20260930</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>AUTOLIV (THAILAND) LIMITED</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>SEAT BELT</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>REQUEST CONTAINER CLEAN &amp; NO SMEL</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>56</v>
+          <t>HASLS22260902044</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>202610040100</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x4 </t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>20260930</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>JINHUA ZINC TECHNOLOGY (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>ZINC OXIDE</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>RQST CONTAINER 30 TONS.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18" ht="13" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902047</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>202610040100</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x4 </t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>20260930</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>JINHUA ZINC TECHNOLOGY (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>ZINC OXIDE</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>RQST CONTAINER 30 TONS.</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="13" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902104</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>202610040100</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>20260930</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>KLOECKNER PENTAPLAST (THAILAND) LTD.</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>DECORATIVE FILMS</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>RQS CLEAN &amp; GOOD CONTAINER CONDITION.</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="13" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902168</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>202610040100</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>KRPUS</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>20261001</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>AUTOLIV (THAILAND) LIMITED</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>SEAT BELT</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>REQUEST CONTAINER CLEAN &amp; NO SMEL</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="13" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902334</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>202610040100</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>20260930</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>BRIDGESTONE TIRE MANUFACTURING (THAILAND) CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>STEEL BOBBINS / PALLET</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="13" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
+      <c r="M22" s="3">
+        <f>SUM(M2:M21)</f>
+        <v/>
+      </c>
+      <c r="N22" s="3">
+        <f>SUM(N2:N21)</f>
+        <v/>
+      </c>
+      <c r="O22" s="3">
+        <f>SUM(O2:O21)</f>
+        <v/>
+      </c>
+      <c r="P22" s="3">
+        <f>SUM(P2:P21)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="3">
+        <f>SUM(Q2:Q21)</f>
+        <v/>
+      </c>
+      <c r="R22" s="3">
+        <f>SUM(R2:R21)</f>
+        <v/>
+      </c>
+      <c r="S22" s="3">
+        <f>SUM(S2:S21)</f>
+        <v/>
+      </c>
+      <c r="T22" s="3">
+        <f>SUM(T2:T21)</f>
+        <v/>
+      </c>
+      <c r="U22" s="3">
+        <f>SUM(U2:U21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="13" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="13" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" ht="13" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>56</v>
+      <c r="B27" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U12"/>
+  <autoFilter ref="A1:U21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update dashboard and reports, merging 9-30-PENDING + 9-30-BKG-3WK
Merged "9-30-PENDING - Copy.xls" (129 new) + "9-30-BKG-3WK -
Copy.xls" (915 new, 2 overlapping) by BK No: 1,044 BK No
outstanding, 2,664 containers. New depot this run: Sintanachote
Co.,Ltd. (9 depots total now). No rows flagged for missing
Pickup Name.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -622,7 +622,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610081000</t>
+          <t>202610082100</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -792,7 +792,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>202610200330</t>
+          <t>202610201730</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -1117,7 +1117,7 @@
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901355</t>
+          <t>HASLS22260901548</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>202610040100</t>
+          <t>202610041200</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>KRKAN</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1153,17 +1153,17 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>20260928</t>
+          <t>20261001</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>HMC POLYMERS CO., LTD.</t>
+          <t>Y-MECO CO., LTD.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>POLYPROPYLENE</t>
+          <t>ASSY COND</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1202,22 +1202,22 @@
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901356</t>
+          <t>HASLS22260901686</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>KXM</t>
+          <t>SWVG</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2608S</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>202610100500</t>
+          <t>202610070330</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -1228,42 +1228,42 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>JPNGO</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx4 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>20261001</t>
+          <t>20261003</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>THAI-YAZAKI ELECTRIC WIRE CO.,LTD.</t>
+          <t>TANATEX CHEMICALS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>COPPER WIRE ROD</t>
+          <t>CHEMICALS PRODUCT DG CARGO</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>REQUEST CONTAINER GRADE A</t>
+          <t>**APPROVAL DG IN SYSTEM DD.24/09/2026** MIX DG22GPx1 (CLS 9 / UN 3082, CLS 8 / UN 3265)</t>
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P9" s="2" t="n">
         <v>0</v>
@@ -1287,7 +1287,7 @@
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901548</t>
+          <t>HASLS22260901795</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>202610040100</t>
+          <t>202610041200</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>KRKAN</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1323,22 +1323,22 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>20261001</t>
+          <t>20260930</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Y-MECO CO., LTD.</t>
+          <t>TRI-WALL PACKAGING (THAI) LTD.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>ASSY COND</t>
+          <t>CORRUGATED PAPER BOARD</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>RQS CLEAN &amp; GOOD CONTAINER CONDITION.</t>
         </is>
       </c>
       <c r="M10" s="2" t="n">
@@ -1372,7 +1372,7 @@
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901686</t>
+          <t>HASLS22260901914</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1398,42 +1398,42 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>JPNGO</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>20260930</t>
+          <t>20260928</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>TANATEX CHEMICALS (THAILAND) CO., LTD.</t>
+          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>CHEMICALS PRODUCT DG CARGO</t>
+          <t>SILICONE</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>**APPROVAL DG IN SYSTEM DD.24/09/2026** MIX DG22GPx1 (CLS 9 / UN 3082, CLS 8 / UN 3265)</t>
+          <t>Good , Clean, No smell container are requested.</t>
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P11" s="2" t="n">
         <v>0</v>
@@ -1457,22 +1457,22 @@
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901795</t>
+          <t>HASLS22260901915</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>KMBK</t>
+          <t>SWVG</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>202610040100</t>
+          <t>202610070330</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1493,22 +1493,22 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>20260930</t>
+          <t>20260928</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>TRI-WALL PACKAGING (THAI) LTD.</t>
+          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>CORRUGATED PAPER BOARD</t>
+          <t>SILICONE</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>RQS CLEAN &amp; GOOD CONTAINER CONDITION.</t>
+          <t>Good , Clean, No smell container are requested.</t>
         </is>
       </c>
       <c r="M12" s="2" t="n">
@@ -1542,22 +1542,22 @@
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901914</t>
+          <t>HASLS22260901971</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>202610070330</t>
+          <t>202610041200</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -1568,42 +1568,42 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>20260928</t>
+          <t>20260930</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
+          <t>BANGKOK CRYSTAL CO., LTD.</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>SILICONE</t>
+          <t>GLASS BLOCK</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Good , Clean, No smell container are requested.</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P13" s="2" t="n">
         <v>0</v>
@@ -1627,22 +1627,22 @@
     <row r="14" ht="13" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901915</t>
+          <t>HASLS22260902009</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>202610070330</t>
+          <t>202610041200</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>KRPUS</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1663,22 +1663,22 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>20260928</t>
+          <t>20260930</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
+          <t>AUTOLIV (THAILAND) LIMITED</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>SILICONE</t>
+          <t>SEAT BELT</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Good , Clean, No smell container are requested.</t>
+          <t>REQUEST CONTAINER CLEAN &amp; NO SMEL</t>
         </is>
       </c>
       <c r="M14" s="2" t="n">
@@ -1712,7 +1712,7 @@
     <row r="15" ht="13" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901971</t>
+          <t>HASLS22260902044</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>202610040100</t>
+          <t>202610041200</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">20'x4 </t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1753,21 +1753,21 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>BANGKOK CRYSTAL CO., LTD.</t>
+          <t>JINHUA ZINC TECHNOLOGY (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>GLASS BLOCK</t>
+          <t>ZINC OXIDE</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>RQST CONTAINER 30 TONS.</t>
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1797,7 +1797,7 @@
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902009</t>
+          <t>HASLS22260902047</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>202610040100</t>
+          <t>202610041200</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
@@ -1823,12 +1823,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>KRPUS</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x4 </t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1838,27 +1838,27 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>AUTOLIV (THAILAND) LIMITED</t>
+          <t>JINHUA ZINC TECHNOLOGY (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>SEAT BELT</t>
+          <t>ZINC OXIDE</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>REQUEST CONTAINER CLEAN &amp; NO SMEL</t>
+          <t>RQST CONTAINER 30 TONS.</t>
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P16" s="2" t="n">
         <v>0</v>
@@ -1882,7 +1882,7 @@
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902044</t>
+          <t>HASLS22260902168</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>202610040100</t>
+          <t>202610041200</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
@@ -1908,42 +1908,42 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>KRPUS</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x4 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>20260930</t>
+          <t>20261001</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>JINHUA ZINC TECHNOLOGY (THAILAND) CO., LTD.</t>
+          <t>AUTOLIV (THAILAND) LIMITED</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>ZINC OXIDE</t>
+          <t>SEAT BELT</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>RQST CONTAINER 30 TONS.</t>
+          <t>REQUEST CONTAINER CLEAN &amp; NO SMEL</t>
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P17" s="2" t="n">
         <v>0</v>
@@ -1967,7 +1967,7 @@
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902047</t>
+          <t>HASLS22260902334</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>202610040100</t>
+          <t>202610041200</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x4 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -2008,27 +2008,27 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>JINHUA ZINC TECHNOLOGY (THAILAND) CO., LTD.</t>
+          <t>BRIDGESTONE TIRE MANUFACTURING (THAILAND) CO.,LTD.</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>ZINC OXIDE</t>
+          <t>STEEL BOBBINS / PALLET</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>RQST CONTAINER 30 TONS.</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P18" s="2" t="n">
         <v>0</v>
@@ -2050,359 +2050,104 @@
       </c>
     </row>
     <row r="19" ht="13" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260902104</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>KMBK</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>202610040100</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>20260930</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>KLOECKNER PENTAPLAST (THAILAND) LTD.</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>DECORATIVE FILMS</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>RQS CLEAN &amp; GOOD CONTAINER CONDITION.</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U19" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="13" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260902168</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>KMBK</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>202610040100</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>20261001</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>AUTOLIV (THAILAND) LIMITED</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>SEAT BELT</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>REQUEST CONTAINER CLEAN &amp; NO SMEL</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U20" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" ht="13" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260902334</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>KMBK</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>202610040100</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40Hx1 </t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>20260930</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>BRIDGESTONE TIRE MANUFACTURING (THAILAND) CO.,LTD.</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>STEEL BOBBINS / PALLET</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U21" s="2" t="n">
-        <v>0</v>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="3">
+        <f>SUM(M2:M18)</f>
+        <v/>
+      </c>
+      <c r="N19" s="3">
+        <f>SUM(N2:N18)</f>
+        <v/>
+      </c>
+      <c r="O19" s="3">
+        <f>SUM(O2:O18)</f>
+        <v/>
+      </c>
+      <c r="P19" s="3">
+        <f>SUM(P2:P18)</f>
+        <v/>
+      </c>
+      <c r="Q19" s="3">
+        <f>SUM(Q2:Q18)</f>
+        <v/>
+      </c>
+      <c r="R19" s="3">
+        <f>SUM(R2:R18)</f>
+        <v/>
+      </c>
+      <c r="S19" s="3">
+        <f>SUM(S2:S18)</f>
+        <v/>
+      </c>
+      <c r="T19" s="3">
+        <f>SUM(T2:T18)</f>
+        <v/>
+      </c>
+      <c r="U19" s="3">
+        <f>SUM(U2:U18)</f>
+        <v/>
       </c>
     </row>
     <row r="22" ht="13" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3">
-        <f>SUM(M2:M21)</f>
-        <v/>
-      </c>
-      <c r="N22" s="3">
-        <f>SUM(N2:N21)</f>
-        <v/>
-      </c>
-      <c r="O22" s="3">
-        <f>SUM(O2:O21)</f>
-        <v/>
-      </c>
-      <c r="P22" s="3">
-        <f>SUM(P2:P21)</f>
-        <v/>
-      </c>
-      <c r="Q22" s="3">
-        <f>SUM(Q2:Q21)</f>
-        <v/>
-      </c>
-      <c r="R22" s="3">
-        <f>SUM(R2:R21)</f>
-        <v/>
-      </c>
-      <c r="S22" s="3">
-        <f>SUM(S2:S21)</f>
-        <v/>
-      </c>
-      <c r="T22" s="3">
-        <f>SUM(T2:T21)</f>
-        <v/>
-      </c>
-      <c r="U22" s="3">
-        <f>SUM(U2:U21)</f>
-        <v/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
       </c>
     </row>
-    <row r="25" ht="13" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
+    <row r="23" ht="13" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>30</v>
       </c>
     </row>
-    <row r="26" ht="13" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="27" ht="13" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="24" ht="13" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>36</v>
+      <c r="B24" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U21"/>
+  <autoFilter ref="A1:U18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update dashboard and reports, merging 10-1-BKG-3WK + 10-1-PENDING
Merged "10-1-BKG-3WK.xls" (924 new) + "10-1-PENDING.xls" (99 new,
no overlap) by BK No: 1,023 BK No outstanding, 2,560 containers,
same 9 depots as yesterday. No rows flagged for missing Pickup
Name.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U24"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -622,7 +622,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610082100</t>
+          <t>202610090100</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -792,7 +792,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>202610201730</t>
+          <t>202610210130</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>202610041200</t>
+          <t>202610040900</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>202610070330</t>
+          <t>202610070430</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -1287,22 +1287,22 @@
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901795</t>
+          <t>HASLS22260901914</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>KMBK</t>
+          <t>SWVG</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>202610041200</t>
+          <t>202610070430</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -1313,32 +1313,32 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>20260930</t>
+          <t>20261001</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>TRI-WALL PACKAGING (THAI) LTD.</t>
+          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>CORRUGATED PAPER BOARD</t>
+          <t>SILICONE</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>RQS CLEAN &amp; GOOD CONTAINER CONDITION.</t>
+          <t>Good , Clean, No smell container are requested.</t>
         </is>
       </c>
       <c r="M10" s="2" t="n">
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P10" s="2" t="n">
         <v>0</v>
@@ -1372,7 +1372,7 @@
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901914</t>
+          <t>HASLS22260901915</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>202610070330</t>
+          <t>202610070430</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>20260928</t>
+          <t>20261002</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1433,7 +1433,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P11" s="2" t="n">
         <v>0</v>
@@ -1457,22 +1457,22 @@
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901915</t>
+          <t>HASLS22260901971</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>202610070330</t>
+          <t>202610040900</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -1483,42 +1483,42 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>20260928</t>
+          <t>20261001</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
+          <t>BANGKOK CRYSTAL CO., LTD.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>SILICONE</t>
+          <t>GLASS BLOCK</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Good , Clean, No smell container are requested.</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P12" s="2" t="n">
         <v>0</v>
@@ -1542,7 +1542,7 @@
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901971</t>
+          <t>HASLS22260902044</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>202610041200</t>
+          <t>202610040900</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">20'x4 </t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1583,17 +1583,17 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>BANGKOK CRYSTAL CO., LTD.</t>
+          <t>JINHUA ZINC TECHNOLOGY (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>GLASS BLOCK</t>
+          <t>ZINC OXIDE</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>RQST CONTAINER 30 TONS.</t>
         </is>
       </c>
       <c r="M13" s="2" t="n">
@@ -1627,7 +1627,7 @@
     <row r="14" ht="13" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902009</t>
+          <t>HASLS22260902168</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>202610041200</t>
+          <t>202610040900</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>20260930</t>
+          <t>20261001</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1710,444 +1710,104 @@
       </c>
     </row>
     <row r="15" ht="13" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260902044</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>KMBK</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>202610041200</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x4 </t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>20260930</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>JINHUA ZINC TECHNOLOGY (THAILAND) CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>ZINC OXIDE</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>RQST CONTAINER 30 TONS.</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" ht="13" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260902047</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>KMBK</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>202610041200</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x4 </t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>20260930</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>JINHUA ZINC TECHNOLOGY (THAILAND) CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>ZINC OXIDE</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>RQST CONTAINER 30 TONS.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U16" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" ht="13" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260902168</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>KMBK</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>202610041200</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40Hx1 </t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>20261001</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>AUTOLIV (THAILAND) LIMITED</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>SEAT BELT</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>REQUEST CONTAINER CLEAN &amp; NO SMEL</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U17" s="2" t="n">
-        <v>0</v>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3">
+        <f>SUM(M2:M14)</f>
+        <v/>
+      </c>
+      <c r="N15" s="3">
+        <f>SUM(N2:N14)</f>
+        <v/>
+      </c>
+      <c r="O15" s="3">
+        <f>SUM(O2:O14)</f>
+        <v/>
+      </c>
+      <c r="P15" s="3">
+        <f>SUM(P2:P14)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="3">
+        <f>SUM(Q2:Q14)</f>
+        <v/>
+      </c>
+      <c r="R15" s="3">
+        <f>SUM(R2:R14)</f>
+        <v/>
+      </c>
+      <c r="S15" s="3">
+        <f>SUM(S2:S14)</f>
+        <v/>
+      </c>
+      <c r="T15" s="3">
+        <f>SUM(T2:T14)</f>
+        <v/>
+      </c>
+      <c r="U15" s="3">
+        <f>SUM(U2:U14)</f>
+        <v/>
       </c>
     </row>
     <row r="18" ht="13" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260902334</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>KMBK</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>202610041200</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>THLCH</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40Hx1 </t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>20260930</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>BRIDGESTONE TIRE MANUFACTURING (THAILAND) CO.,LTD.</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>STEEL BOBBINS / PALLET</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U18" s="2" t="n">
-        <v>0</v>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="13" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="n"/>
-      <c r="M19" s="3">
-        <f>SUM(M2:M18)</f>
-        <v/>
-      </c>
-      <c r="N19" s="3">
-        <f>SUM(N2:N18)</f>
-        <v/>
-      </c>
-      <c r="O19" s="3">
-        <f>SUM(O2:O18)</f>
-        <v/>
-      </c>
-      <c r="P19" s="3">
-        <f>SUM(P2:P18)</f>
-        <v/>
-      </c>
-      <c r="Q19" s="3">
-        <f>SUM(Q2:Q18)</f>
-        <v/>
-      </c>
-      <c r="R19" s="3">
-        <f>SUM(R2:R18)</f>
-        <v/>
-      </c>
-      <c r="S19" s="3">
-        <f>SUM(S2:S18)</f>
-        <v/>
-      </c>
-      <c r="T19" s="3">
-        <f>SUM(T2:T18)</f>
-        <v/>
-      </c>
-      <c r="U19" s="3">
-        <f>SUM(U2:U18)</f>
-        <v/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>21</v>
       </c>
     </row>
-    <row r="22" ht="13" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="13" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="24" ht="13" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="20" ht="13" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>30</v>
+      <c r="B20" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U18"/>
+  <autoFilter ref="A1:U14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update reports with 10-2-BKG-3-5-OCT + 10-2-PD; prefer standard 27-col sheet
Merged "10-2-BKG-3-5-OCT.xls" (121 new) + "10-2-PD.xls" (80 new, PD
last) by BK No: 201 BK No outstanding, 596 containers, 6 depots,
no missing Pickup Name.

10-2-PD.xls had three sheets: one with embedded duplicate headers,
one with a duplicated ETD column (28 cols) and a blank Return
header, and one standard 27-col sheet. _pick_clean_sheet() now
breaks ties on duplicate-header count by closeness to the standard
27 columns, so the standard sheet is chosen and the merge header
check passes.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -607,22 +607,22 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802361</t>
+          <t>HASLS22260802276</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SWRG</t>
+          <t>SWAT</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610131130</t>
+          <t>202610090100</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -633,27 +633,27 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>JPTYO</t>
+          <t>TWKEL</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx3 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>20260923</t>
+          <t>20261003</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>L. LIGHTING GLASS CO., LTD.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>GLASS TUBES FOR ELECTRIC LIGHTING</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -662,13 +662,13 @@
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>0</v>
@@ -707,7 +707,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>202610131130</t>
+          <t>202610141700</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -828,7 +828,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>REQ GOOD AND CLEAN CONTAINER</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
@@ -862,22 +862,22 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901914</t>
+          <t>HASLS22260901089</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>KUS</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2616N</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>202610070830</t>
+          <t>202610150400</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -888,42 +888,42 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>JPIYM</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>20261001</t>
+          <t>20261005</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>SHIN-ETSU SILICONES (THAILAND) LTD.</t>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>SILICONE</t>
+          <t>RESIN</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Good , Clean, No smell container are requested.</t>
+          <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P5" s="2" t="n">
         <v>0</v>
@@ -945,104 +945,189 @@
       </c>
     </row>
     <row r="6" ht="13" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260901686</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>202610070930</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>JPNGO</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>20261003</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>TANATEX CHEMICALS (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>CHEMICALS PRODUCT DG CARGO</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>**APPROVAL DG IN SYSTEM DD.24/09/2026** MIX DG22GPx1 (CLS 9 / UN 3082, CLS 8 / UN 3265)</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="13" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3">
-        <f>SUM(M2:M5)</f>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3">
+        <f>SUM(M2:M6)</f>
         <v/>
       </c>
-      <c r="N6" s="3">
-        <f>SUM(N2:N5)</f>
+      <c r="N7" s="3">
+        <f>SUM(N2:N6)</f>
         <v/>
       </c>
-      <c r="O6" s="3">
-        <f>SUM(O2:O5)</f>
+      <c r="O7" s="3">
+        <f>SUM(O2:O6)</f>
         <v/>
       </c>
-      <c r="P6" s="3">
-        <f>SUM(P2:P5)</f>
+      <c r="P7" s="3">
+        <f>SUM(P2:P6)</f>
         <v/>
       </c>
-      <c r="Q6" s="3">
-        <f>SUM(Q2:Q5)</f>
+      <c r="Q7" s="3">
+        <f>SUM(Q2:Q6)</f>
         <v/>
       </c>
-      <c r="R6" s="3">
-        <f>SUM(R2:R5)</f>
+      <c r="R7" s="3">
+        <f>SUM(R2:R6)</f>
         <v/>
       </c>
-      <c r="S6" s="3">
-        <f>SUM(S2:S5)</f>
+      <c r="S7" s="3">
+        <f>SUM(S2:S6)</f>
         <v/>
       </c>
-      <c r="T6" s="3">
-        <f>SUM(T2:T5)</f>
+      <c r="T7" s="3">
+        <f>SUM(T2:T6)</f>
         <v/>
       </c>
-      <c r="U6" s="3">
-        <f>SUM(U2:U5)</f>
+      <c r="U7" s="3">
+        <f>SUM(U2:U6)</f>
         <v/>
-      </c>
-    </row>
-    <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
       </c>
     </row>
     <row r="10" ht="13" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>8</v>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
       </c>
     </row>
     <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" ht="13" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>8</v>
+      <c r="B12" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U5"/>
+  <autoFilter ref="A1:U6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update reports with 10-5-BKG-3WK + 10-5-PENDING
Merged "10-5-BKG-3WK.xls" (1,014 new) + "10-5-PENDING.xls" (76 new,
PENDING last) by BK No, no overlap: 1,090 BK No outstanding, 2,876
containers across 8 depots (Sintanachote and UNITHAI back). One row
flagged for missing Pickup Name: HASLS22260900416 (the same BK No
flagged repeatedly in earlier runs).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -658,7 +658,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
@@ -692,12 +692,12 @@
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900838</t>
+          <t>HASLS22260802485</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SWRG</t>
+          <t>HMVY</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>202610141700</t>
+          <t>202610201100</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -718,22 +718,22 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>JPNAH</t>
+          <t>JPIYM</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>20260930</t>
+          <t>20261007</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>THAI POLYETHYLENE CO., LTD.</t>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -743,11 +743,11 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>RESIN-PALLET,NO RED WALL CONTAINER,CLEAN CONTAINER NO OIL STAINS , NO RUSTY ,NO CUT OR HOLE</t>
+          <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>0</v>
@@ -777,22 +777,22 @@
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900975</t>
+          <t>HASLS22260900838</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>KMSU</t>
+          <t>SWRG</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2608S</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>202610251730</t>
+          <t>202610141700</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -803,7 +803,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>JPNAH</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -818,17 +818,17 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>TANATEX CHEMICALS (THAILAND) CO., LTD.</t>
+          <t>THAI POLYETHYLENE CO., LTD.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>CHEMICALS PRODUCT (NON DG)</t>
+          <t>RESIN</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>RESIN-PALLET,NO RED WALL CONTAINER,CLEAN CONTAINER NO OIL STAINS , NO RUSTY ,NO CUT OR HOLE</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
@@ -862,22 +862,22 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901089</t>
+          <t>HASLS22260900975</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>KUS</t>
+          <t>KMSU</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2616N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>202610150400</t>
+          <t>202610251730</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -888,36 +888,36 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>20261005</t>
+          <t>20260930</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>TANATEX CHEMICALS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>CHEMICALS PRODUCT (NON DG)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -947,22 +947,22 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901686</t>
+          <t>HASLS22260901089</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SWVG</t>
+          <t>KUS</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2616N</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>202610070930</t>
+          <t>202610150400</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -973,7 +973,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>JPNGO</t>
+          <t>JPIYM</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -983,22 +983,22 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>20261003</t>
+          <t>20261005</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>TANATEX CHEMICALS (THAILAND) CO., LTD.</t>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>CHEMICALS PRODUCT DG CARGO</t>
+          <t>RESIN</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>**APPROVAL DG IN SYSTEM DD.24/09/2026** MIX DG22GPx1 (CLS 9 / UN 3082, CLS 8 / UN 3265)</t>
+          <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
@@ -1030,104 +1030,444 @@
       </c>
     </row>
     <row r="7" ht="13" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3">
-        <f>SUM(M2:M6)</f>
-        <v/>
-      </c>
-      <c r="N7" s="3">
-        <f>SUM(N2:N6)</f>
-        <v/>
-      </c>
-      <c r="O7" s="3">
-        <f>SUM(O2:O6)</f>
-        <v/>
-      </c>
-      <c r="P7" s="3">
-        <f>SUM(P2:P6)</f>
-        <v/>
-      </c>
-      <c r="Q7" s="3">
-        <f>SUM(Q2:Q6)</f>
-        <v/>
-      </c>
-      <c r="R7" s="3">
-        <f>SUM(R2:R6)</f>
-        <v/>
-      </c>
-      <c r="S7" s="3">
-        <f>SUM(S2:S6)</f>
-        <v/>
-      </c>
-      <c r="T7" s="3">
-        <f>SUM(T2:T6)</f>
-        <v/>
-      </c>
-      <c r="U7" s="3">
-        <f>SUM(U2:U6)</f>
-        <v/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902842</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>KUS</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2617N</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>202611041300</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x9 </t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>20261022</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="13" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902847</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>202610250700</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x4 </t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>20261019</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="13" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902848</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>202610250700</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x2 </t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>20261019</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="13" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22261000207</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>HMVY</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>202610201100</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>JPIYM</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>20261007</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
+      <c r="M11" s="3">
+        <f>SUM(M2:M10)</f>
+        <v/>
+      </c>
+      <c r="N11" s="3">
+        <f>SUM(N2:N10)</f>
+        <v/>
+      </c>
+      <c r="O11" s="3">
+        <f>SUM(O2:O10)</f>
+        <v/>
+      </c>
+      <c r="P11" s="3">
+        <f>SUM(P2:P10)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="3">
+        <f>SUM(Q2:Q10)</f>
+        <v/>
+      </c>
+      <c r="R11" s="3">
+        <f>SUM(R2:R10)</f>
+        <v/>
+      </c>
+      <c r="S11" s="3">
+        <f>SUM(S2:S10)</f>
+        <v/>
+      </c>
+      <c r="T11" s="3">
+        <f>SUM(T2:T10)</f>
+        <v/>
+      </c>
+      <c r="U11" s="3">
+        <f>SUM(U2:U10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="13" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="13" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>CELLO</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>7</v>
+      <c r="B15" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>23</v>
       </c>
     </row>
-    <row r="12" ht="13" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="16" ht="13" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>7</v>
+      <c r="B16" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U6"/>
+  <autoFilter ref="A1:U10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update reports with 10-6-BKG-3WK + 10-6-PENDING
Merged "10-6-BKG-3WK.xls" (1,032 new) + "10-6-PENDING.xls" (91 new,
1 overlapping, PENDING last) by BK No: 1,122 BK No outstanding,
2,987 containers across 9 depots (ICD LKT back). One row flagged
for missing Pickup Name: HASLS22261000388 (MARINE EXPRESS CO., LTD.,
1 container) — a different BK No from the one already excluded.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -607,22 +607,22 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260802276</t>
+          <t>HASLS22260802147</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SWAT</t>
+          <t>SWSR</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610090100</t>
+          <t>202610130600</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -633,42 +633,42 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>TWKEL</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>20261003</t>
+          <t>20261009</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>L. LIGHTING GLASS CO., LTD.</t>
+          <t>CHIBA METAL (THAILAND) CO.,LTD</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>GLASS TUBES FOR ELECTRIC LIGHTING</t>
+          <t xml:space="preserve">ELECTRONIC PART/TERMINAL/MICROSPEAKER </t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>good, clean, dry, no leak, no hole</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>0</v>
@@ -777,22 +777,22 @@
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900838</t>
+          <t>HASLS22260900975</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SWRG</t>
+          <t>KMSU</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>202610141700</t>
+          <t>202610280830</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -803,7 +803,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>JPNAH</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -818,17 +818,17 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>THAI POLYETHYLENE CO., LTD.</t>
+          <t>TANATEX CHEMICALS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>CHEMICALS PRODUCT (NON DG)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>RESIN-PALLET,NO RED WALL CONTAINER,CLEAN CONTAINER NO OIL STAINS , NO RUSTY ,NO CUT OR HOLE</t>
+          <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
@@ -862,22 +862,22 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900975</t>
+          <t>HASLS22260901089</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>KMSU</t>
+          <t>KUS</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2608S</t>
+          <t>2616N</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>202610251730</t>
+          <t>202610150400</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -888,36 +888,36 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>JPIYM</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>20260930</t>
+          <t>20261005</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>TANATEX CHEMICALS (THAILAND) CO., LTD.</t>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>CHEMICALS PRODUCT (NON DG)</t>
+          <t>RESIN</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>GOOD AND CLEAN CTNR</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -947,12 +947,12 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901089</t>
+          <t>HASLS22260902087</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>KUS</t>
+          <t>SWBT</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>202610150400</t>
+          <t>202610161500</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -973,42 +973,42 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>20261005</t>
+          <t>20261009</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>SENNICS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>SIRANTOX 6PPD(4020)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>GOOD DRY AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P6" s="2" t="n">
         <v>0</v>
@@ -1032,22 +1032,22 @@
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902842</t>
+          <t>HASLS22260902231</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>KUS</t>
+          <t>PCCP</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2617N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>202611041300</t>
+          <t>202610121600</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -1063,37 +1063,37 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x9 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>20261022</t>
+          <t>20261007</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>TRI-WALL PACKAGING (THAI) LTD.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>CORRUGATED PAPER BOARD</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>RQS CLEAN &amp; GOOD CONTAINER CONDITION.</t>
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P7" s="2" t="n">
         <v>0</v>
@@ -1117,12 +1117,12 @@
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902847</t>
+          <t>HASLS22260902603</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>KMBK</t>
+          <t>KMTP</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>202610250700</t>
+          <t>202610150800</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -1143,42 +1143,42 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNXMN</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x4 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>20261019</t>
+          <t>20261007</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+          <t>SADESA (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>RESIN</t>
+          <t>COW LEATHER (DRY SKIN)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CTNR</t>
+          <t>REQUEST CONTAINER: NO LEAK,NO HOLE,CLEAN</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8" s="2" t="n">
         <v>0</v>
@@ -1202,22 +1202,22 @@
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902848</t>
+          <t>HASLS22260902842</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>KMBK</t>
+          <t>KUS</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2617N</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>202610250700</t>
+          <t>202611041300</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -1233,12 +1233,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">20'x9 </t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>20261019</t>
+          <t>20261022</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -1287,22 +1287,22 @@
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000207</t>
+          <t>HASLS22260902847</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>HMVY</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>202610201100</t>
+          <t>202610250700</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -1313,17 +1313,17 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>JPIYM</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx4 </t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>20261007</t>
+          <t>20261019</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1342,13 +1342,13 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P10" s="2" t="n">
         <v>0</v>
@@ -1370,104 +1370,529 @@
       </c>
     </row>
     <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3">
-        <f>SUM(M2:M10)</f>
-        <v/>
-      </c>
-      <c r="N11" s="3">
-        <f>SUM(N2:N10)</f>
-        <v/>
-      </c>
-      <c r="O11" s="3">
-        <f>SUM(O2:O10)</f>
-        <v/>
-      </c>
-      <c r="P11" s="3">
-        <f>SUM(P2:P10)</f>
-        <v/>
-      </c>
-      <c r="Q11" s="3">
-        <f>SUM(Q2:Q10)</f>
-        <v/>
-      </c>
-      <c r="R11" s="3">
-        <f>SUM(R2:R10)</f>
-        <v/>
-      </c>
-      <c r="S11" s="3">
-        <f>SUM(S2:S10)</f>
-        <v/>
-      </c>
-      <c r="T11" s="3">
-        <f>SUM(T2:T10)</f>
-        <v/>
-      </c>
-      <c r="U11" s="3">
-        <f>SUM(U2:U10)</f>
-        <v/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902848</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>202610250700</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x2 </t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>20261019</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="13" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902849</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>PGPO</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>202610160200</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>20261009</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>SENNICS (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>SIRANTOX 6PPD(4020)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>GOOD DRY AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="13" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902851</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SWIC</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>202610152200</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx4 </t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>20261008</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>TOSHIBA CONSUMER PRODUCTS (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>WASHING MACHINE</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14" ht="13" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22261000031</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>PGPO</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>202610160200</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>KRINC</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>20261008</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>ASIAN HONDA MOTOR CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>SPARE PARTS FOR HONDA MOTORCYCLES,SPARE PARTS FOR HONDA AUTOMOBILES</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>**APPROVAL BY MR.LEE MINHA DD.02/10/2026**  DG45GPx1 (CLS 8 / UN 2800)</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="13" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>23</v>
+          <t>HASLS22261000207</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>HMVY</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>202610201100</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>JPIYM</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>20261007</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="n"/>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3">
+        <f>SUM(M2:M15)</f>
+        <v/>
+      </c>
+      <c r="N16" s="3">
+        <f>SUM(N2:N15)</f>
+        <v/>
+      </c>
+      <c r="O16" s="3">
+        <f>SUM(O2:O15)</f>
+        <v/>
+      </c>
+      <c r="P16" s="3">
+        <f>SUM(P2:P15)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="3">
+        <f>SUM(Q2:Q15)</f>
+        <v/>
+      </c>
+      <c r="R16" s="3">
+        <f>SUM(R2:R15)</f>
+        <v/>
+      </c>
+      <c r="S16" s="3">
+        <f>SUM(S2:S15)</f>
+        <v/>
+      </c>
+      <c r="T16" s="3">
+        <f>SUM(T2:T15)</f>
+        <v/>
+      </c>
+      <c r="U16" s="3">
+        <f>SUM(U2:U15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="13" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="13" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" ht="13" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>23</v>
+      <c r="B21" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U10"/>
+  <autoFilter ref="A1:U15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update reports with 10-22-PD data
Regenerated from the full daily export "10-22-PD.xls" (3,143
rows): 78 BK No outstanding, 251 containers across 7 depots (TIFFA
LOGISTICS CENTER appears this run). No rows flagged for missing
Pickup Name.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - CELLO.xlsx
+++ b/output/bkg pending - CELLO.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -607,7 +607,7 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000016</t>
+          <t>HASLS22260900467</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202611041200</t>
+          <t>202611082100</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -638,12 +638,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx4 </t>
+          <t xml:space="preserve">40Hx6 </t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>20261021</t>
+          <t>20261022</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -690,104 +690,274 @@
       </c>
     </row>
     <row r="3" ht="13" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22261000016</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>SWSP</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>202611082100</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx4 </t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>20261021</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="13" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22261001160</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SWSP</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>202611082100</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x2 </t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>20261022</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>PTT GLOBAL CHEMICAL PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>RESIN</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CTNR</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="13" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3">
-        <f>SUM(M2:M2)</f>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3">
+        <f>SUM(M2:M4)</f>
         <v/>
       </c>
-      <c r="N3" s="3">
-        <f>SUM(N2:N2)</f>
+      <c r="N5" s="3">
+        <f>SUM(N2:N4)</f>
         <v/>
       </c>
-      <c r="O3" s="3">
-        <f>SUM(O2:O2)</f>
+      <c r="O5" s="3">
+        <f>SUM(O2:O4)</f>
         <v/>
       </c>
-      <c r="P3" s="3">
-        <f>SUM(P2:P2)</f>
+      <c r="P5" s="3">
+        <f>SUM(P2:P4)</f>
         <v/>
       </c>
-      <c r="Q3" s="3">
-        <f>SUM(Q2:Q2)</f>
+      <c r="Q5" s="3">
+        <f>SUM(Q2:Q4)</f>
         <v/>
       </c>
-      <c r="R3" s="3">
-        <f>SUM(R2:R2)</f>
+      <c r="R5" s="3">
+        <f>SUM(R2:R4)</f>
         <v/>
       </c>
-      <c r="S3" s="3">
-        <f>SUM(S2:S2)</f>
+      <c r="S5" s="3">
+        <f>SUM(S2:S4)</f>
         <v/>
       </c>
-      <c r="T3" s="3">
-        <f>SUM(T2:T2)</f>
+      <c r="T5" s="3">
+        <f>SUM(T2:T4)</f>
         <v/>
       </c>
-      <c r="U3" s="3">
-        <f>SUM(U2:U2)</f>
+      <c r="U5" s="3">
+        <f>SUM(U2:U4)</f>
         <v/>
-      </c>
-    </row>
-    <row r="6" ht="13" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="13" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>CELLO</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="8" ht="13" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="13" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>CELLO</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" ht="13" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>4</v>
+      <c r="B10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U2"/>
+  <autoFilter ref="A1:U4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>